<commit_message>
1. Updated the features 2. Updated test data sheet 3. Fix the failed scripts
</commit_message>
<xml_diff>
--- a/data/CPSUI_Automation_Data.xlsx
+++ b/data/CPSUI_Automation_Data.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="10956" windowHeight="7692" tabRatio="933" activeTab="5"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="10956" windowHeight="7692" tabRatio="933" firstSheet="5" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="PhoneSearch" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="893" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="891" uniqueCount="240">
   <si>
     <t>Update and validate the phone number preferences</t>
   </si>
@@ -649,9 +649,6 @@
     <t>HRS</t>
   </si>
   <si>
-    <t>01/25/21</t>
-  </si>
-  <si>
     <t>01/25/2021</t>
   </si>
   <si>
@@ -673,12 +670,6 @@
     <t>R10 Member Portal</t>
   </si>
   <si>
-    <t>AF45799</t>
-  </si>
-  <si>
-    <t>11/02/2020</t>
-  </si>
-  <si>
     <t>KS0763929</t>
   </si>
   <si>
@@ -752,9 +743,6 @@
   </si>
   <si>
     <t>Error messages validation in email history search screen</t>
-  </si>
-  <si>
-    <t>//scenarios_data_files//dummyTestt.txt</t>
   </si>
   <si>
     <t>345 6454 544</t>
@@ -771,6 +759,15 @@
   </si>
   <si>
     <t>5/13/2021</t>
+  </si>
+  <si>
+    <t>SMC_BATCH</t>
+  </si>
+  <si>
+    <t>04/29/2021</t>
+  </si>
+  <si>
+    <t>01/25/21</t>
   </si>
 </sst>
 </file>
@@ -1253,7 +1250,7 @@
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -1266,7 +1263,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>1</v>
@@ -1300,7 +1297,7 @@
         <v>0</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>2</v>
@@ -1435,7 +1432,8 @@
     <col min="18" max="18" width="10.21875" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="12" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="25.44140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="22" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.3">
@@ -1497,7 +1495,7 @@
         <v>135</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="U1" s="2" t="s">
         <v>15</v>
@@ -1538,7 +1536,7 @@
         <v>75</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="L2" s="6" t="s">
         <v>93</v>
@@ -1558,16 +1556,16 @@
         <v>199</v>
       </c>
       <c r="S2" s="9" t="s">
+        <v>239</v>
+      </c>
+      <c r="T2" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="T2" s="9" t="s">
-        <v>201</v>
-      </c>
       <c r="U2" s="9" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="V2" s="9" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.3">
@@ -1584,23 +1582,23 @@
         <v>62</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="5" t="s">
         <v>205</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>206</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>87</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="K3" s="1" t="s">
         <v>202</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>203</v>
       </c>
       <c r="L3" s="6">
         <v>20</v>
@@ -1634,23 +1632,23 @@
         <v>62</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="5" t="s">
         <v>205</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>206</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>87</v>
       </c>
       <c r="I4" s="1"/>
       <c r="J4" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="K4" s="1" t="s">
         <v>202</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>203</v>
       </c>
       <c r="L4" s="6">
         <v>20</v>
@@ -1792,23 +1790,23 @@
         <v>62</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="5" t="s">
         <v>205</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>206</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>87</v>
       </c>
       <c r="I2" s="1"/>
       <c r="J2" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2" s="1" t="s">
         <v>202</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>203</v>
       </c>
       <c r="L2" s="6">
         <v>20</v>
@@ -1820,14 +1818,14 @@
         <v>2010313141</v>
       </c>
       <c r="O2" s="5" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="P2" s="5"/>
       <c r="Q2" s="5" t="s">
-        <v>208</v>
+        <v>237</v>
       </c>
       <c r="R2" s="20" t="s">
-        <v>209</v>
+        <v>238</v>
       </c>
       <c r="S2" s="6"/>
       <c r="T2" s="6"/>
@@ -1865,7 +1863,7 @@
         <v>75</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="L3" s="6" t="s">
         <v>93</v>
@@ -1877,10 +1875,10 @@
       <c r="Q3" s="5"/>
       <c r="R3" s="3"/>
       <c r="S3" s="6" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="T3" s="6" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="U3" s="6"/>
     </row>
@@ -1889,7 +1887,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>62</v>
@@ -1916,7 +1914,7 @@
         <v>75</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="L4" s="6" t="s">
         <v>93</v>
@@ -1936,7 +1934,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>62</v>
@@ -1963,7 +1961,7 @@
         <v>75</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="L5" s="6" t="s">
         <v>93</v>
@@ -1981,7 +1979,7 @@
         <v>163</v>
       </c>
       <c r="U5" s="1" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.3">
@@ -1989,7 +1987,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>62</v>
@@ -2016,7 +2014,7 @@
         <v>75</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="L6" s="6" t="s">
         <v>93</v>
@@ -2034,7 +2032,7 @@
         <v>25</v>
       </c>
       <c r="U6" s="1" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.3">
@@ -2042,7 +2040,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>62</v>
@@ -2069,7 +2067,7 @@
         <v>75</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="L7" s="6" t="s">
         <v>93</v>
@@ -2087,7 +2085,7 @@
         <v>25</v>
       </c>
       <c r="U7" s="1" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.3">
@@ -2095,7 +2093,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>62</v>
@@ -2122,7 +2120,7 @@
         <v>75</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="L8" s="6" t="s">
         <v>93</v>
@@ -2140,7 +2138,7 @@
         <v>28</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.3">
@@ -2148,7 +2146,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>62</v>
@@ -2175,7 +2173,7 @@
         <v>75</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="L9" s="6" t="s">
         <v>93</v>
@@ -2195,7 +2193,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>62</v>
@@ -2204,23 +2202,23 @@
         <v>62</v>
       </c>
       <c r="E10" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="5" t="s">
         <v>205</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>206</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>87</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="K10" s="1" t="s">
         <v>202</v>
-      </c>
-      <c r="K10" s="1" t="s">
-        <v>203</v>
       </c>
       <c r="L10" s="6">
         <v>20</v>
@@ -2307,8 +2305,8 @@
       <c r="B2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="22" t="s">
-        <v>236</v>
+      <c r="C2" s="22">
+        <v>3456454544</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>1</v>
@@ -2328,7 +2326,7 @@
         <v>13</v>
       </c>
       <c r="C3" s="22">
-        <v>7579.3433340000001</v>
+        <v>7579343334</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>1</v>
@@ -2347,8 +2345,8 @@
       <c r="B4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="22" t="s">
-        <v>237</v>
+      <c r="C4" s="22">
+        <v>6175057744</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>2</v>
@@ -2433,10 +2431,10 @@
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="F8" s="3" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="H8" s="1"/>
     </row>
@@ -2614,7 +2612,7 @@
         <v>35</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>235</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -2797,14 +2795,14 @@
         <v>77</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="K3" s="1"/>
       <c r="L3" s="6">
@@ -3764,16 +3762,16 @@
       </c>
       <c r="V2" s="5"/>
       <c r="W2" s="5" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="X2" s="9" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="Y2" s="9" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="Z2" s="9" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.3">
@@ -4096,7 +4094,7 @@
         <v>150</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="S2" s="1" t="s">
         <v>88</v>
@@ -4251,7 +4249,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>62</v>
@@ -4316,7 +4314,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>62</v>
@@ -4381,7 +4379,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>62</v>
@@ -4446,7 +4444,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>62</v>
@@ -4497,7 +4495,7 @@
         <v>28</v>
       </c>
       <c r="AA8" s="1" t="s">
-        <v>23</v>
+        <v>230</v>
       </c>
       <c r="AB8" s="1"/>
       <c r="AC8" s="1"/>
@@ -4511,7 +4509,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>62</v>
@@ -4570,7 +4568,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>62</v>
@@ -5188,7 +5186,7 @@
         <v>28</v>
       </c>
       <c r="AG19" s="1" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
     </row>
     <row r="21" spans="1:33" x14ac:dyDescent="0.3">
@@ -5319,7 +5317,7 @@
         <v>195</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="T1" s="2" t="s">
         <v>102</v>
@@ -5378,7 +5376,7 @@
         <v>75</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="L2" s="6" t="s">
         <v>93</v>
@@ -5387,7 +5385,7 @@
         <v>193</v>
       </c>
       <c r="N2" s="8" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="O2" s="6" t="s">
         <v>194</v>
@@ -5400,10 +5398,10 @@
         <v>196</v>
       </c>
       <c r="S2" s="5" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="T2" s="8" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="U2" s="5" t="s">
         <v>107</v>
@@ -5415,16 +5413,16 @@
         <v>150</v>
       </c>
       <c r="X2" s="9" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="Y2" s="9" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="Z2" s="9" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="AA2" s="9" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.3">
@@ -5441,20 +5439,20 @@
         <v>62</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>87</v>
       </c>
       <c r="I3" s="5"/>
       <c r="J3" s="1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="K3" s="1">
         <v>493364140</v>

</xml_diff>

<commit_message>
1. Added the more data's in scenario outline
2. Updated the data sheet with new combinations
</commit_message>
<xml_diff>
--- a/data/CPSUI_Automation_Data.xlsx
+++ b/data/CPSUI_Automation_Data.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="10956" windowHeight="7692" tabRatio="933" firstSheet="5" activeTab="9"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="10956" windowHeight="7692" tabRatio="933"/>
   </bookViews>
   <sheets>
     <sheet name="PhoneSearch" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="891" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="981" uniqueCount="256">
   <si>
     <t>Update and validate the phone number preferences</t>
   </si>
@@ -768,6 +768,54 @@
   </si>
   <si>
     <t>01/25/21</t>
+  </si>
+  <si>
+    <t>827T61169</t>
+  </si>
+  <si>
+    <t>RHONDA</t>
+  </si>
+  <si>
+    <t>HANSON</t>
+  </si>
+  <si>
+    <t>03/01/1978</t>
+  </si>
+  <si>
+    <t>00188703</t>
+  </si>
+  <si>
+    <t>DONALD</t>
+  </si>
+  <si>
+    <t>DONALDSON</t>
+  </si>
+  <si>
+    <t>07/18/1962</t>
+  </si>
+  <si>
+    <t>CLIFFORD</t>
+  </si>
+  <si>
+    <t>EDWARDS</t>
+  </si>
+  <si>
+    <t>09/30/1944</t>
+  </si>
+  <si>
+    <t>Georgia</t>
+  </si>
+  <si>
+    <t>617T95817</t>
+  </si>
+  <si>
+    <t>NIGIDAN</t>
+  </si>
+  <si>
+    <t>RAVI</t>
+  </si>
+  <si>
+    <t>02/08/1940</t>
   </si>
 </sst>
 </file>
@@ -1410,7 +1458,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:V9"/>
+  <dimension ref="A1:V11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.6640625" bestFit="1" customWidth="1"/>
@@ -1668,13 +1716,213 @@
       <c r="U4" s="6"/>
       <c r="V4" s="6"/>
     </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="K5" s="1">
+        <v>245687858</v>
+      </c>
+      <c r="L5" s="6">
+        <v>10</v>
+      </c>
+      <c r="M5" s="6"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="1"/>
+      <c r="P5" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="R5" s="6"/>
+      <c r="S5" s="6"/>
+      <c r="T5" s="6"/>
+      <c r="U5" s="6"/>
+      <c r="V5" s="6"/>
+    </row>
+    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="K6" s="1">
+        <v>245687858</v>
+      </c>
+      <c r="L6" s="6">
+        <v>10</v>
+      </c>
+      <c r="M6" s="6"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
+      <c r="P6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q6" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="R6" s="6"/>
+      <c r="S6" s="6"/>
+      <c r="T6" s="6"/>
+      <c r="U6" s="6"/>
+      <c r="V6" s="6"/>
+    </row>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="M7" s="6"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q7" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
+      <c r="U7" s="6"/>
+      <c r="V7" s="6"/>
+    </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="B8" t="s">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="L8" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="M8" s="6"/>
+      <c r="N8" s="1"/>
+      <c r="O8" s="1"/>
+      <c r="P8" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="R8" s="6"/>
+      <c r="S8" s="6"/>
+      <c r="T8" s="6"/>
+      <c r="U8" s="6"/>
+      <c r="V8" s="6"/>
+    </row>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="B10" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="B9" t="s">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="B11" t="s">
         <v>121</v>
       </c>
     </row>
@@ -3595,7 +3843,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Z9"/>
+  <dimension ref="A1:Z11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.6640625" bestFit="1" customWidth="1"/>
@@ -3615,7 +3863,7 @@
     <col min="15" max="15" width="13.44140625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="13.5546875" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="9.21875" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="29" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="11.5546875" bestFit="1" customWidth="1"/>
@@ -3886,13 +4134,237 @@
       <c r="Y4" s="6"/>
       <c r="Z4" s="6"/>
     </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="L5" s="6">
+        <v>1</v>
+      </c>
+      <c r="M5" s="6"/>
+      <c r="N5" s="6"/>
+      <c r="O5" s="6"/>
+      <c r="P5" s="1"/>
+      <c r="Q5" s="1"/>
+      <c r="R5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="S5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="T5" s="6"/>
+      <c r="U5" s="6"/>
+      <c r="V5" s="6"/>
+      <c r="W5" s="6"/>
+      <c r="X5" s="6"/>
+      <c r="Y5" s="6"/>
+      <c r="Z5" s="6"/>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="L6" s="6">
+        <v>1</v>
+      </c>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="1"/>
+      <c r="Q6" s="1"/>
+      <c r="R6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="S6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="T6" s="6"/>
+      <c r="U6" s="6"/>
+      <c r="V6" s="6"/>
+      <c r="W6" s="6"/>
+      <c r="X6" s="6"/>
+      <c r="Y6" s="6"/>
+      <c r="Z6" s="6"/>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>247</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="I7" s="6">
+        <v>270000</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="K7" s="1">
+        <v>269648884</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="1"/>
+      <c r="Q7" s="1"/>
+      <c r="R7" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="S7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="T7" s="6"/>
+      <c r="U7" s="6"/>
+      <c r="V7" s="6"/>
+      <c r="W7" s="6"/>
+      <c r="X7" s="6"/>
+      <c r="Y7" s="6"/>
+      <c r="Z7" s="6"/>
+    </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="B8" t="s">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>247</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="I8" s="6">
+        <v>270000</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="K8" s="1">
+        <v>269648884</v>
+      </c>
+      <c r="L8" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="M8" s="6"/>
+      <c r="N8" s="6"/>
+      <c r="O8" s="6"/>
+      <c r="P8" s="1"/>
+      <c r="Q8" s="1"/>
+      <c r="R8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="S8" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="T8" s="6"/>
+      <c r="U8" s="6"/>
+      <c r="V8" s="6"/>
+      <c r="W8" s="6"/>
+      <c r="X8" s="6"/>
+      <c r="Y8" s="6"/>
+      <c r="Z8" s="6"/>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="B10" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="B9" t="s">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="B11" t="s">
         <v>121</v>
       </c>
     </row>

</xml_diff>

<commit_message>
1. Updated the test data sheet.
2. Changed the ie options for driver.

3. Added the OS property in extent.properties. By this, we can see the
OS in extent reports.

4. Updated the IEDriver to 3.15 version

5. Added the dependency for javax.mail for SMTP

6. Called the triggerMail method under @AfterClass hook in both
Runner.java and RunnerForFailedScenarios.java classes. So once the
execution is completed the mail will be sent to the recipients.

7.  Created a new class to send the mail with extent report. This class
works by using java mail API and more details mentioned inside class.
</commit_message>
<xml_diff>
--- a/data/CPSUI_Automation_Data.xlsx
+++ b/data/CPSUI_Automation_Data.xlsx
@@ -3,13 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="164011"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AG53052\EclipseWorkspace\CPSUI_Automation\Data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="10956" windowHeight="7692" tabRatio="933"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22152" windowHeight="8340" tabRatio="786" firstSheet="6" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="PhoneSearch" sheetId="1" r:id="rId1"/>
@@ -24,7 +19,8 @@
     <sheet name="GovtMemberContactInfPhone" sheetId="10" r:id="rId10"/>
     <sheet name="Govt_Mbr_Text_Mail_Email_Pref" sheetId="11" r:id="rId11"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1:M27"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="981" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="986" uniqueCount="259">
   <si>
     <t>Update and validate the phone number preferences</t>
   </si>
@@ -770,21 +766,6 @@
     <t>01/25/21</t>
   </si>
   <si>
-    <t>827T61169</t>
-  </si>
-  <si>
-    <t>RHONDA</t>
-  </si>
-  <si>
-    <t>HANSON</t>
-  </si>
-  <si>
-    <t>03/01/1978</t>
-  </si>
-  <si>
-    <t>00188703</t>
-  </si>
-  <si>
     <t>DONALD</t>
   </si>
   <si>
@@ -806,16 +787,40 @@
     <t>Georgia</t>
   </si>
   <si>
-    <t>617T95817</t>
-  </si>
-  <si>
-    <t>NIGIDAN</t>
-  </si>
-  <si>
-    <t>RAVI</t>
-  </si>
-  <si>
-    <t>02/08/1940</t>
+    <t>01/01/1980</t>
+  </si>
+  <si>
+    <t>JOAN</t>
+  </si>
+  <si>
+    <t>KS0802408</t>
+  </si>
+  <si>
+    <t>ARD</t>
+  </si>
+  <si>
+    <t>05/24/2010</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> comment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">should be last updated by TINA </t>
+  </si>
+  <si>
+    <t>ELIZABETH</t>
+  </si>
+  <si>
+    <t>702T93657</t>
+  </si>
+  <si>
+    <t>ROSSI03</t>
+  </si>
+  <si>
+    <t>VALENTINO03</t>
+  </si>
+  <si>
+    <t>10/22/1934</t>
   </si>
 </sst>
 </file>
@@ -884,7 +889,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -907,11 +912,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -955,6 +971,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1244,7 +1263,7 @@
     <col min="2" max="2" width="50.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="37.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
@@ -1263,6 +1282,9 @@
       <c r="E1" s="2" t="s">
         <v>7</v>
       </c>
+      <c r="F1" s="23" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
@@ -1429,13 +1451,15 @@
         <v>10</v>
       </c>
       <c r="C12" s="22">
-        <v>2694895564</v>
+        <v>4556864560</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E12" s="1"/>
-      <c r="F12" s="21"/>
+      <c r="F12" s="21" t="s">
+        <v>253</v>
+      </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
@@ -1630,26 +1654,26 @@
         <v>62</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>203</v>
+        <v>254</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>204</v>
+        <v>250</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>205</v>
+        <v>251</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>87</v>
+        <v>192</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="1" t="s">
-        <v>201</v>
+        <v>75</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="L3" s="6">
-        <v>20</v>
+        <v>249</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>93</v>
       </c>
       <c r="M3" s="6"/>
       <c r="N3" s="1"/>
@@ -1680,26 +1704,26 @@
         <v>62</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>203</v>
+        <v>254</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>204</v>
+        <v>250</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>205</v>
+        <v>251</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>87</v>
+        <v>192</v>
       </c>
       <c r="I4" s="1"/>
       <c r="J4" s="1" t="s">
-        <v>201</v>
+        <v>75</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="L4" s="6">
-        <v>20</v>
+        <v>249</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>93</v>
       </c>
       <c r="M4" s="6"/>
       <c r="N4" s="1"/>
@@ -1730,16 +1754,16 @@
         <v>62</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="I5" s="1"/>
       <c r="J5" s="1" t="s">
@@ -1780,16 +1804,16 @@
         <v>62</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="1" t="s">
@@ -1830,23 +1854,23 @@
         <v>62</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>255</v>
+        <v>257</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>258</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>192</v>
+        <v>87</v>
       </c>
       <c r="I7" s="1"/>
       <c r="J7" s="1" t="s">
         <v>67</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="L7" s="6" t="s">
         <v>71</v>
@@ -1880,23 +1904,23 @@
         <v>62</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>255</v>
+        <v>257</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>258</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>192</v>
+        <v>87</v>
       </c>
       <c r="I8" s="1"/>
       <c r="J8" s="1" t="s">
         <v>67</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="L8" s="6" t="s">
         <v>71</v>
@@ -2450,26 +2474,26 @@
         <v>62</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>203</v>
+        <v>254</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>204</v>
+        <v>250</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>205</v>
+        <v>251</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>87</v>
+        <v>192</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1" t="s">
-        <v>201</v>
+        <v>75</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="L10" s="6">
-        <v>20</v>
+        <v>249</v>
+      </c>
+      <c r="L10" s="6" t="s">
+        <v>93</v>
       </c>
       <c r="M10" s="6"/>
       <c r="N10" s="6"/>
@@ -4148,28 +4172,28 @@
         <v>62</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>242</v>
+        <v>81</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>244</v>
+        <v>82</v>
+      </c>
+      <c r="I5" s="5">
+        <v>174134</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="L5" s="6">
-        <v>1</v>
+        <v>74</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>93</v>
       </c>
       <c r="M5" s="6"/>
       <c r="N5" s="6"/>
@@ -4204,28 +4228,28 @@
         <v>62</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>242</v>
+        <v>81</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>244</v>
+        <v>82</v>
+      </c>
+      <c r="I6" s="5">
+        <v>174134</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="L6" s="6">
-        <v>1</v>
+        <v>74</v>
+      </c>
+      <c r="L6" s="6" t="s">
+        <v>93</v>
       </c>
       <c r="M6" s="6"/>
       <c r="N6" s="6"/>
@@ -4260,13 +4284,13 @@
         <v>62</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>119</v>
@@ -4316,13 +4340,13 @@
         <v>62</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>119</v>

</xml_diff>

<commit_message>
1. Scripts are failing in IE browser because of locators. So changed some of the locators CSS selectors and modified the xPath's of some locators.
2. Modified the sorting methods. Earlier, sorting will happen once the
PEGA_GRID value changes only. But now sorting will happen once the table
refresh is completed.

3. Updated the data sheet. Changed the path of file locations and couple
of headers.

4. Added a recipient in sendReport class.

5.  Created couple of reusable methods in utils class and modified
getText() method.
</commit_message>
<xml_diff>
--- a/data/CPSUI_Automation_Data.xlsx
+++ b/data/CPSUI_Automation_Data.xlsx
@@ -3,8 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="164011"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AG53052\EclipseWorkspace\CPSUI_Automation\Data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22152" windowHeight="8340" tabRatio="786" firstSheet="6" activeTab="9"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22152" windowHeight="8340" tabRatio="786" firstSheet="7" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="PhoneSearch" sheetId="1" r:id="rId1"/>
@@ -20,7 +25,6 @@
     <sheet name="Govt_Mbr_Text_Mail_Email_Pref" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:M27"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -134,9 +138,6 @@
     <t>Sales</t>
   </si>
   <si>
-    <t>//scenarios_data_files//dummyTest.txt</t>
-  </si>
-  <si>
     <t>Non-sales</t>
   </si>
   <si>
@@ -180,9 +181,6 @@
   </si>
   <si>
     <t>create a consent or do not call or wrong number file with more than  20000 phone numbers</t>
-  </si>
-  <si>
-    <t>//scenarios_data_files//UAT_Morethan_20000.txt</t>
   </si>
   <si>
     <t>Search the member by using wildcard search</t>
@@ -821,6 +819,12 @@
   </si>
   <si>
     <t>10/22/1934</t>
+  </si>
+  <si>
+    <t>\scenarios_data_files\dummyTest.txt</t>
+  </si>
+  <si>
+    <t>\scenarios_data_files\UAT_Morethan_20000.txt</t>
   </si>
 </sst>
 </file>
@@ -1283,7 +1287,7 @@
         <v>7</v>
       </c>
       <c r="F1" s="23" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -1320,7 +1324,7 @@
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -1333,7 +1337,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>1</v>
@@ -1367,7 +1371,7 @@
         <v>0</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>2</v>
@@ -1458,7 +1462,7 @@
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="21" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -1516,43 +1520,43 @@
         <v>4</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>61</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="P1" s="2" t="s">
         <v>6</v>
@@ -1561,13 +1565,13 @@
         <v>7</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="U1" s="2" t="s">
         <v>15</v>
@@ -1581,37 +1585,37 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>190</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>192</v>
       </c>
       <c r="I2" s="1">
         <v>186100</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M2" s="5">
         <v>7858408019</v>
@@ -1625,19 +1629,19 @@
       <c r="P2" s="5"/>
       <c r="Q2" s="5"/>
       <c r="R2" s="5" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="S2" s="9" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="T2" s="9" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="U2" s="9" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="V2" s="9" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.3">
@@ -1645,35 +1649,35 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M3" s="6"/>
       <c r="N3" s="1"/>
@@ -1695,35 +1699,35 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="I4" s="1"/>
       <c r="J4" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M4" s="6"/>
       <c r="N4" s="1"/>
@@ -1745,29 +1749,29 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="G5" s="5" t="s">
         <v>243</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>244</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>245</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>246</v>
       </c>
       <c r="I5" s="1"/>
       <c r="J5" s="1" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="K5" s="1">
         <v>245687858</v>
@@ -1795,29 +1799,29 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E6" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>243</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>244</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>245</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>246</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="1" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="K6" s="1">
         <v>245687858</v>
@@ -1845,35 +1849,35 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="G7" s="3" t="s">
         <v>256</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>257</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>258</v>
-      </c>
       <c r="H7" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="I7" s="1"/>
       <c r="J7" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M7" s="6"/>
       <c r="N7" s="1"/>
@@ -1895,35 +1899,35 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E8" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="G8" s="3" t="s">
         <v>256</v>
       </c>
-      <c r="F8" s="1" t="s">
-        <v>257</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>258</v>
-      </c>
       <c r="H8" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="I8" s="1"/>
       <c r="J8" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M8" s="6"/>
       <c r="N8" s="1"/>
@@ -1942,12 +1946,12 @@
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -1991,61 +1995,61 @@
         <v>4</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="K1" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>61</v>
-      </c>
       <c r="M1" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="N1" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="O1" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="N1" s="12" t="s">
+      <c r="P1" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="O1" s="12" t="s">
+      <c r="Q1" s="12" t="s">
         <v>139</v>
       </c>
-      <c r="P1" s="12" t="s">
+      <c r="R1" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="Q1" s="12" t="s">
-        <v>141</v>
-      </c>
-      <c r="R1" s="12" t="s">
-        <v>142</v>
-      </c>
       <c r="S1" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="T1" s="17" t="s">
+        <v>177</v>
+      </c>
+      <c r="U1" s="17" t="s">
         <v>178</v>
-      </c>
-      <c r="T1" s="17" t="s">
-        <v>179</v>
-      </c>
-      <c r="U1" s="17" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.3">
@@ -2053,51 +2057,51 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>205</v>
-      </c>
       <c r="H2" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="I2" s="1"/>
       <c r="J2" s="1" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="L2" s="6">
         <v>20</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N2" s="5">
         <v>2010313141</v>
       </c>
       <c r="O2" s="5" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="P2" s="5"/>
       <c r="Q2" s="5" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="R2" s="20" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="S2" s="6"/>
       <c r="T2" s="6"/>
@@ -2108,37 +2112,37 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>190</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>192</v>
       </c>
       <c r="I3" s="1">
         <v>186100</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M3" s="6"/>
       <c r="N3" s="5"/>
@@ -2147,10 +2151,10 @@
       <c r="Q3" s="5"/>
       <c r="R3" s="3"/>
       <c r="S3" s="6" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="T3" s="6" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="U3" s="6"/>
     </row>
@@ -2159,37 +2163,37 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="G4" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>190</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>192</v>
       </c>
       <c r="I4" s="1">
         <v>186100</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M4" s="6"/>
       <c r="N4" s="5"/>
@@ -2206,37 +2210,37 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="G5" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>190</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>192</v>
       </c>
       <c r="I5" s="1">
         <v>186100</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M5" s="6"/>
       <c r="N5" s="5"/>
@@ -2245,13 +2249,13 @@
       <c r="Q5" s="5"/>
       <c r="R5" s="3"/>
       <c r="S5" s="3" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="T5" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="U5" s="1" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.3">
@@ -2259,37 +2263,37 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E6" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>190</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>192</v>
       </c>
       <c r="I6" s="1">
         <v>186100</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M6" s="6"/>
       <c r="N6" s="5"/>
@@ -2304,7 +2308,7 @@
         <v>25</v>
       </c>
       <c r="U6" s="1" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.3">
@@ -2312,37 +2316,37 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>190</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>192</v>
       </c>
       <c r="I7" s="1">
         <v>186100</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M7" s="6"/>
       <c r="N7" s="5"/>
@@ -2357,7 +2361,7 @@
         <v>25</v>
       </c>
       <c r="U7" s="1" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.3">
@@ -2365,37 +2369,37 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E8" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="G8" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="H8" s="1" t="s">
         <v>190</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>192</v>
       </c>
       <c r="I8" s="1">
         <v>186100</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M8" s="6"/>
       <c r="N8" s="6"/>
@@ -2410,7 +2414,7 @@
         <v>28</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.3">
@@ -2418,37 +2422,37 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E9" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="H9" s="1" t="s">
         <v>190</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>192</v>
       </c>
       <c r="I9" s="1">
         <v>186100</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M9" s="6"/>
       <c r="N9" s="6"/>
@@ -2465,35 +2469,35 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M10" s="6"/>
       <c r="N10" s="6"/>
@@ -2507,24 +2511,24 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A14" s="15"/>
       <c r="B14" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A15" s="16"/>
       <c r="B15" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -2703,10 +2707,10 @@
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="F8" s="3" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="H8" s="1"/>
     </row>
@@ -2816,7 +2820,7 @@
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -2850,7 +2854,7 @@
         <v>30</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -2867,7 +2871,7 @@
         <v>33</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>34</v>
+        <v>257</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -2881,10 +2885,10 @@
         <v>32</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>34</v>
+        <v>257</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -2895,13 +2899,13 @@
         <v>31</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>34</v>
+        <v>257</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -2909,7 +2913,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>32</v>
@@ -2924,13 +2928,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>32</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E6" s="1"/>
     </row>
@@ -2939,13 +2943,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E7" s="1"/>
     </row>
@@ -2981,34 +2985,34 @@
         <v>4</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
@@ -3016,35 +3020,35 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E2" s="1" t="s">
+      <c r="G2" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>64</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>66</v>
       </c>
       <c r="I2" s="1"/>
       <c r="J2" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
@@ -3052,29 +3056,29 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="1" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="K3" s="1"/>
       <c r="L3" s="6">
@@ -3086,35 +3090,35 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="H4" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>82</v>
       </c>
       <c r="I4" s="1"/>
       <c r="J4" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
@@ -3122,35 +3126,35 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="G5" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>86</v>
-      </c>
       <c r="H5" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I5" s="1"/>
       <c r="J5" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="K5" s="1">
         <v>233866906</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
@@ -3158,7 +3162,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
@@ -3169,7 +3173,7 @@
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L6" s="6"/>
     </row>
@@ -3178,7 +3182,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -3189,7 +3193,7 @@
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="L7" s="6"/>
     </row>
@@ -3198,7 +3202,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
@@ -3209,7 +3213,7 @@
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="L8" s="6"/>
     </row>
@@ -3218,7 +3222,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
@@ -3238,7 +3242,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -3248,7 +3252,7 @@
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
       <c r="J10" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="K10" s="1">
         <v>123456789</v>
@@ -3257,12 +3261,12 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -3294,13 +3298,13 @@
         <v>30</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>41</v>
-      </c>
       <c r="F1" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -3308,7 +3312,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>33</v>
@@ -3317,10 +3321,10 @@
         <v>2</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>34</v>
+        <v>257</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -3328,19 +3332,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>34</v>
+        <v>257</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -3348,19 +3352,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>34</v>
+        <v>257</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -3368,19 +3372,19 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>34</v>
+        <v>257</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -3388,19 +3392,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>34</v>
+        <v>257</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3408,7 +3412,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>33</v>
@@ -3417,7 +3421,7 @@
         <v>2</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F7" s="1"/>
     </row>
@@ -3426,16 +3430,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>1</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F8" s="1"/>
     </row>
@@ -3444,16 +3448,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F9" s="1"/>
     </row>
@@ -3462,16 +3466,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F10" s="1"/>
     </row>
@@ -3480,16 +3484,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F11" s="1"/>
     </row>
@@ -3498,7 +3502,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>33</v>
@@ -3507,10 +3511,10 @@
         <v>2</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>50</v>
+        <v>258</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -3518,19 +3522,19 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>1</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>50</v>
+        <v>258</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
@@ -3538,19 +3542,19 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>50</v>
+        <v>258</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -3558,19 +3562,19 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>50</v>
+        <v>258</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -3578,19 +3582,19 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>50</v>
+        <v>258</v>
       </c>
     </row>
   </sheetData>
@@ -3640,73 +3644,73 @@
         <v>4</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="K1" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>61</v>
-      </c>
       <c r="M1" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="R1" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="N1" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="Q1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="R1" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="S1" s="2" t="s">
+      <c r="T1" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="U1" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="U1" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="V1" s="2" t="s">
-        <v>105</v>
-      </c>
       <c r="W1" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="X1" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="Y1" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="Z1" s="2" t="s">
         <v>15</v>
@@ -3720,80 +3724,80 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E2" s="1" t="s">
+      <c r="G2" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>92</v>
-      </c>
       <c r="H2" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="I2" s="1">
         <v>174134</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K2" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="M2" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="N2" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="L2" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="M2" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="N2" s="8" t="s">
-        <v>96</v>
-      </c>
       <c r="O2" s="6" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="P2" s="8">
         <v>8185555555</v>
       </c>
       <c r="Q2" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="R2" s="5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="S2" s="5" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="T2" s="5"/>
       <c r="U2" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="V2" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="W2" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="V2" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="W2" s="5" t="s">
-        <v>108</v>
-      </c>
       <c r="X2" s="9" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="Y2" s="9" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="Z2" s="9" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="AA2" s="9" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.3">
@@ -3801,34 +3805,34 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E3" s="1" t="s">
+      <c r="G3" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="H3" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>120</v>
-      </c>
       <c r="J3" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="L3" s="6">
         <v>2</v>
@@ -3851,12 +3855,12 @@
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -3904,49 +3908,49 @@
         <v>4</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="K1" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>61</v>
-      </c>
       <c r="M1" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="O1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="R1" s="2" t="s">
         <v>6</v>
@@ -3955,19 +3959,19 @@
         <v>7</v>
       </c>
       <c r="T1" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="W1" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="U1" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="V1" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="W1" s="2" t="s">
-        <v>136</v>
-      </c>
       <c r="X1" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="Y1" s="2" t="s">
         <v>15</v>
@@ -3981,41 +3985,41 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>92</v>
-      </c>
       <c r="H2" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="I2" s="1">
         <v>174134</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M2" s="6"/>
       <c r="N2" s="5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="O2" s="5">
         <v>8185555555</v>
@@ -4030,20 +4034,20 @@
       <c r="S2" s="5"/>
       <c r="T2" s="5"/>
       <c r="U2" s="11" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="V2" s="5"/>
       <c r="W2" s="5" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="X2" s="9" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="Y2" s="9" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="Z2" s="9" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.3">
@@ -4051,34 +4055,34 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="H3" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>120</v>
-      </c>
       <c r="J3" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="L3" s="6">
         <v>2</v>
@@ -4107,34 +4111,34 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G4" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="I4" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="H4" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>120</v>
-      </c>
       <c r="J4" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="L4" s="6">
         <v>2</v>
@@ -4163,37 +4167,37 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="I5" s="5">
         <v>174134</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M5" s="6"/>
       <c r="N5" s="6"/>
@@ -4219,37 +4223,37 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="I6" s="5">
         <v>174134</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M6" s="6"/>
       <c r="N6" s="6"/>
@@ -4275,37 +4279,37 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>241</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>242</v>
-      </c>
       <c r="H7" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="I7" s="6">
         <v>270000</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K7" s="1">
         <v>269648884</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M7" s="6"/>
       <c r="N7" s="6"/>
@@ -4331,37 +4335,37 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E8" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="G8" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="F8" s="1" t="s">
-        <v>241</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>242</v>
-      </c>
       <c r="H8" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="I8" s="6">
         <v>270000</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K8" s="1">
         <v>269648884</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M8" s="6"/>
       <c r="N8" s="6"/>
@@ -4384,12 +4388,12 @@
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -4444,97 +4448,97 @@
         <v>4</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="K1" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>61</v>
-      </c>
       <c r="M1" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="N1" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="O1" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="N1" s="12" t="s">
+      <c r="P1" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="O1" s="12" t="s">
+      <c r="Q1" s="12" t="s">
         <v>139</v>
       </c>
-      <c r="P1" s="12" t="s">
+      <c r="R1" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="Q1" s="12" t="s">
+      <c r="S1" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="R1" s="12" t="s">
+      <c r="T1" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="U1" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="S1" s="13" t="s">
+      <c r="V1" s="13" t="s">
         <v>143</v>
       </c>
-      <c r="T1" s="13" t="s">
-        <v>148</v>
-      </c>
-      <c r="U1" s="13" t="s">
+      <c r="W1" s="13" t="s">
         <v>144</v>
       </c>
-      <c r="V1" s="13" t="s">
+      <c r="X1" s="13" t="s">
         <v>145</v>
       </c>
-      <c r="W1" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="X1" s="13" t="s">
-        <v>147</v>
-      </c>
       <c r="Y1" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="Z1" s="17" t="s">
+        <v>177</v>
+      </c>
+      <c r="AA1" s="17" t="s">
         <v>178</v>
       </c>
-      <c r="Z1" s="17" t="s">
+      <c r="AB1" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="AC1" s="19" t="s">
+        <v>166</v>
+      </c>
+      <c r="AD1" s="19" t="s">
+        <v>163</v>
+      </c>
+      <c r="AE1" s="19" t="s">
+        <v>174</v>
+      </c>
+      <c r="AF1" s="19" t="s">
+        <v>175</v>
+      </c>
+      <c r="AG1" s="19" t="s">
         <v>179</v>
-      </c>
-      <c r="AA1" s="17" t="s">
-        <v>180</v>
-      </c>
-      <c r="AB1" s="19" t="s">
-        <v>167</v>
-      </c>
-      <c r="AC1" s="19" t="s">
-        <v>168</v>
-      </c>
-      <c r="AD1" s="19" t="s">
-        <v>165</v>
-      </c>
-      <c r="AE1" s="19" t="s">
-        <v>176</v>
-      </c>
-      <c r="AF1" s="19" t="s">
-        <v>177</v>
-      </c>
-      <c r="AG1" s="19" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="2" spans="1:33" x14ac:dyDescent="0.3">
@@ -4542,71 +4546,71 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>92</v>
-      </c>
       <c r="H2" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="I2" s="1">
         <v>174134</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N2" s="5">
         <v>5139699786</v>
       </c>
       <c r="O2" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="P2" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="Q2" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="T2" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="Q2" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="R2" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="T2" s="6" t="s">
-        <v>151</v>
-      </c>
       <c r="U2" s="6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="V2" s="6"/>
       <c r="W2" s="6" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="X2" s="6" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="Y2" s="6"/>
       <c r="Z2" s="6"/>
@@ -4623,37 +4627,37 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>92</v>
-      </c>
       <c r="H3" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="I3" s="1">
         <v>174134</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M3" s="6"/>
       <c r="N3" s="5"/>
@@ -4668,10 +4672,10 @@
       <c r="W3" s="6"/>
       <c r="X3" s="6"/>
       <c r="Y3" s="6" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="Z3" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="AA3" s="6"/>
       <c r="AB3" s="1"/>
@@ -4686,34 +4690,34 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G4" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="I4" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="H4" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>120</v>
-      </c>
       <c r="J4" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="L4" s="6">
         <v>2</v>
@@ -4745,37 +4749,37 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G5" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>92</v>
-      </c>
       <c r="H5" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="I5" s="1">
         <v>174134</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M5" s="6"/>
       <c r="N5" s="5"/>
@@ -4790,13 +4794,13 @@
       <c r="W5" s="6"/>
       <c r="X5" s="6"/>
       <c r="Y5" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="Z5" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="AA5" s="1" t="s">
         <v>162</v>
-      </c>
-      <c r="Z5" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="AA5" s="1" t="s">
-        <v>164</v>
       </c>
       <c r="AB5" s="1"/>
       <c r="AC5" s="1"/>
@@ -4810,37 +4814,37 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E6" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>92</v>
-      </c>
       <c r="H6" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="I6" s="1">
         <v>174134</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M6" s="6"/>
       <c r="N6" s="5"/>
@@ -4875,37 +4879,37 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>92</v>
-      </c>
       <c r="H7" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="I7" s="1">
         <v>174134</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M7" s="6"/>
       <c r="N7" s="5"/>
@@ -4940,37 +4944,37 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E8" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G8" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="F8" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>92</v>
-      </c>
       <c r="H8" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="I8" s="1">
         <v>174134</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M8" s="6"/>
       <c r="N8" s="6"/>
@@ -4991,7 +4995,7 @@
         <v>28</v>
       </c>
       <c r="AA8" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="AB8" s="1"/>
       <c r="AC8" s="1"/>
@@ -5005,37 +5009,37 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E9" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="F9" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>92</v>
-      </c>
       <c r="H9" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="I9" s="1">
         <v>174134</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M9" s="6"/>
       <c r="N9" s="6"/>
@@ -5064,34 +5068,34 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E10" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G10" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="H10" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="I10" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="H10" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>120</v>
-      </c>
       <c r="J10" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="L10" s="6">
         <v>2</v>
@@ -5123,37 +5127,37 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E11" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G11" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="F11" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>92</v>
-      </c>
       <c r="H11" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="I11" s="1">
         <v>174134</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M11" s="6"/>
       <c r="N11" s="6"/>
@@ -5182,34 +5186,34 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E12" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G12" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="H12" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="I12" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="H12" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="I12" s="5" t="s">
-        <v>120</v>
-      </c>
       <c r="J12" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="L12" s="6">
         <v>2</v>
@@ -5241,37 +5245,37 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E13" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G13" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="F13" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>92</v>
-      </c>
       <c r="H13" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="I13" s="1">
         <v>174134</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M13" s="6"/>
       <c r="N13" s="6"/>
@@ -5289,13 +5293,13 @@
       <c r="Z13" s="3"/>
       <c r="AA13" s="1"/>
       <c r="AB13" s="1" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="AC13" s="1" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="AD13" s="1" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="AE13" s="1"/>
       <c r="AF13" s="1"/>
@@ -5306,34 +5310,34 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E14" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G14" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="H14" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G14" s="5" t="s">
+      <c r="I14" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="H14" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="I14" s="5" t="s">
-        <v>120</v>
-      </c>
       <c r="J14" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="L14" s="6">
         <v>2</v>
@@ -5357,10 +5361,10 @@
       <c r="AC14" s="1"/>
       <c r="AD14" s="1"/>
       <c r="AE14" s="5" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="AF14" s="5" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="AG14" s="1"/>
     </row>
@@ -5369,34 +5373,34 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E15" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G15" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="H15" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G15" s="5" t="s">
+      <c r="I15" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="H15" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="I15" s="5" t="s">
-        <v>120</v>
-      </c>
       <c r="J15" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="L15" s="6">
         <v>2</v>
@@ -5422,7 +5426,7 @@
       <c r="AE15" s="1"/>
       <c r="AF15" s="1"/>
       <c r="AG15" s="1" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="16" spans="1:33" x14ac:dyDescent="0.3">
@@ -5430,34 +5434,34 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E16" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G16" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="H16" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G16" s="5" t="s">
+      <c r="I16" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="H16" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="I16" s="5" t="s">
-        <v>120</v>
-      </c>
       <c r="J16" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="L16" s="6">
         <v>2</v>
@@ -5481,13 +5485,13 @@
       <c r="AC16" s="1"/>
       <c r="AD16" s="1"/>
       <c r="AE16" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="AF16" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="AG16" s="1" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="17" spans="1:33" x14ac:dyDescent="0.3">
@@ -5495,34 +5499,34 @@
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E17" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G17" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="H17" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G17" s="5" t="s">
+      <c r="I17" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="H17" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="I17" s="5" t="s">
-        <v>120</v>
-      </c>
       <c r="J17" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="L17" s="6">
         <v>2</v>
@@ -5560,34 +5564,34 @@
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E18" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G18" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="H18" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G18" s="5" t="s">
+      <c r="I18" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="H18" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="I18" s="5" t="s">
-        <v>120</v>
-      </c>
       <c r="J18" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="L18" s="6">
         <v>2</v>
@@ -5617,7 +5621,7 @@
         <v>25</v>
       </c>
       <c r="AG18" s="1" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="19" spans="1:33" x14ac:dyDescent="0.3">
@@ -5625,34 +5629,34 @@
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E19" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G19" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="H19" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G19" s="5" t="s">
+      <c r="I19" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="H19" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="I19" s="5" t="s">
-        <v>120</v>
-      </c>
       <c r="J19" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="L19" s="6">
         <v>2</v>
@@ -5682,41 +5686,41 @@
         <v>28</v>
       </c>
       <c r="AG19" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="21" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="22" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="23" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A23" s="15"/>
       <c r="B23" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="24" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A24" s="14"/>
       <c r="B24" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="25" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A25" s="16"/>
       <c r="B25" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="26" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A26" s="18"/>
       <c r="B26" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -5753,8 +5757,8 @@
     <col min="23" max="23" width="10.21875" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="39.33203125" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="32.21875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="22.44140625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="21.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.3">
@@ -5765,79 +5769,79 @@
         <v>4</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="K1" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>61</v>
-      </c>
       <c r="M1" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="O1" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="Q1" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="P1" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="T1" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="R1" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="T1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="U1" s="2" t="s">
-        <v>104</v>
-      </c>
       <c r="V1" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="W1" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="X1" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="Y1" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="Z1" s="2" t="s">
-        <v>15</v>
+        <v>176</v>
       </c>
       <c r="AA1" s="2" t="s">
-        <v>16</v>
+        <v>177</v>
       </c>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.3">
@@ -5845,80 +5849,80 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>190</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>192</v>
       </c>
       <c r="I2" s="1">
         <v>186100</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M2" s="10" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="N2" s="8" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="O2" s="6" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="P2" s="8">
         <v>7858408019</v>
       </c>
       <c r="Q2" s="5"/>
       <c r="R2" s="5" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="S2" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="T2" s="8" t="s">
         <v>209</v>
       </c>
-      <c r="T2" s="8" t="s">
+      <c r="U2" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="V2" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="W2" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="X2" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="Y2" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="Z2" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="U2" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="V2" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="W2" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="X2" s="9" t="s">
-        <v>212</v>
-      </c>
-      <c r="Y2" s="9" t="s">
-        <v>212</v>
-      </c>
-      <c r="Z2" s="9" t="s">
-        <v>213</v>
-      </c>
       <c r="AA2" s="9" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.3">
@@ -5926,29 +5930,29 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="I3" s="5"/>
       <c r="J3" s="1" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="K3" s="1">
         <v>493364140</v>
@@ -5974,12 +5978,12 @@
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
As part of PEGA upgrade, most of the locators are changed. So updated the locators from id to xPath and used contains mostly in xPath's.
1. Update the locators in page object classes.

2. Changed the error messages in feature files.

3. Added assert.fail() method in existing util methods.
</commit_message>
<xml_diff>
--- a/data/CPSUI_Automation_Data.xlsx
+++ b/data/CPSUI_Automation_Data.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22152" windowHeight="8340" tabRatio="786" firstSheet="7" activeTab="8"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22152" windowHeight="8340" tabRatio="786" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="PhoneSearch" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="986" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="986" uniqueCount="257">
   <si>
     <t>Update and validate the phone number preferences</t>
   </si>
@@ -535,9 +535,6 @@
     <t>5/16/2020</t>
   </si>
   <si>
-    <t>History Details:Please enter From Date and End Date within 1 year range.</t>
-  </si>
-  <si>
     <t>messageInPreferenceTab</t>
   </si>
   <si>
@@ -595,9 +592,6 @@
     <t>4/20/2021</t>
   </si>
   <si>
-    <t>Commercial Member:Please enter From Date and End Date within 1 year range.</t>
-  </si>
-  <si>
     <t>No Records found for the input criteria</t>
   </si>
   <si>
@@ -698,18 +692,6 @@
   </si>
   <si>
     <t>4/22/2021</t>
-  </si>
-  <si>
-    <t>History Details:Please enter From Date and End Date within 6 months range.</t>
-  </si>
-  <si>
-    <t>** End Date must not be greater than current date.</t>
-  </si>
-  <si>
-    <t>** From Date must not be greater than current date.</t>
-  </si>
-  <si>
-    <t>** The From Date must come before the End Date.</t>
   </si>
   <si>
     <t>WAWID062</t>
@@ -825,6 +807,18 @@
   </si>
   <si>
     <t>\scenarios_data_files\UAT_Morethan_20000.txt</t>
+  </si>
+  <si>
+    <t>Commercial Member: Please enter From Date and End Date within 1 year range.</t>
+  </si>
+  <si>
+    <t>History Details: Please enter From Date and End Date within 6 months range.</t>
+  </si>
+  <si>
+    <t>End Date must not be greater than current date.</t>
+  </si>
+  <si>
+    <t>History Details: Please enter From Date and End Date within 1 year range.</t>
   </si>
 </sst>
 </file>
@@ -1287,7 +1281,7 @@
         <v>7</v>
       </c>
       <c r="F1" s="23" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -1324,7 +1318,7 @@
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -1337,7 +1331,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>1</v>
@@ -1371,7 +1365,7 @@
         <v>0</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>2</v>
@@ -1462,7 +1456,7 @@
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="21" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -1571,7 +1565,7 @@
         <v>133</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="U1" s="2" t="s">
         <v>15</v>
@@ -1585,7 +1579,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>60</v>
@@ -1594,16 +1588,16 @@
         <v>60</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>188</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>190</v>
       </c>
       <c r="I2" s="1">
         <v>186100</v>
@@ -1612,7 +1606,7 @@
         <v>73</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="L2" s="6" t="s">
         <v>91</v>
@@ -1629,19 +1623,19 @@
       <c r="P2" s="5"/>
       <c r="Q2" s="5"/>
       <c r="R2" s="5" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="S2" s="9" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="T2" s="9" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="U2" s="9" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="V2" s="9" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.3">
@@ -1649,7 +1643,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>60</v>
@@ -1658,23 +1652,23 @@
         <v>60</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="1" t="s">
         <v>73</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="L3" s="6" t="s">
         <v>91</v>
@@ -1699,7 +1693,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>60</v>
@@ -1708,23 +1702,23 @@
         <v>60</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="I4" s="1"/>
       <c r="J4" s="1" t="s">
         <v>73</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="L4" s="6" t="s">
         <v>91</v>
@@ -1749,7 +1743,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>60</v>
@@ -1758,20 +1752,20 @@
         <v>60</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="I5" s="1"/>
       <c r="J5" s="1" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="K5" s="1">
         <v>245687858</v>
@@ -1799,7 +1793,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>60</v>
@@ -1808,20 +1802,20 @@
         <v>60</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="1" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="K6" s="1">
         <v>245687858</v>
@@ -1849,7 +1843,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>60</v>
@@ -1858,13 +1852,13 @@
         <v>60</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>85</v>
@@ -1874,7 +1868,7 @@
         <v>65</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="L7" s="6" t="s">
         <v>69</v>
@@ -1899,7 +1893,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>60</v>
@@ -1908,13 +1902,13 @@
         <v>60</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>85</v>
@@ -1924,7 +1918,7 @@
         <v>65</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="L8" s="6" t="s">
         <v>69</v>
@@ -2043,13 +2037,13 @@
         <v>140</v>
       </c>
       <c r="S1" s="17" t="s">
+        <v>175</v>
+      </c>
+      <c r="T1" s="17" t="s">
         <v>176</v>
       </c>
-      <c r="T1" s="17" t="s">
+      <c r="U1" s="17" t="s">
         <v>177</v>
-      </c>
-      <c r="U1" s="17" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.3">
@@ -2066,23 +2060,23 @@
         <v>60</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>201</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>203</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>85</v>
       </c>
       <c r="I2" s="1"/>
       <c r="J2" s="1" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="L2" s="6">
         <v>20</v>
@@ -2094,14 +2088,14 @@
         <v>2010313141</v>
       </c>
       <c r="O2" s="5" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="P2" s="5"/>
       <c r="Q2" s="5" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="R2" s="20" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="S2" s="6"/>
       <c r="T2" s="6"/>
@@ -2121,16 +2115,16 @@
         <v>60</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>188</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>190</v>
       </c>
       <c r="I3" s="1">
         <v>186100</v>
@@ -2139,7 +2133,7 @@
         <v>73</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="L3" s="6" t="s">
         <v>91</v>
@@ -2151,10 +2145,10 @@
       <c r="Q3" s="5"/>
       <c r="R3" s="3"/>
       <c r="S3" s="6" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="T3" s="6" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="U3" s="6"/>
     </row>
@@ -2163,7 +2157,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>60</v>
@@ -2172,16 +2166,16 @@
         <v>60</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="G4" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>188</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>190</v>
       </c>
       <c r="I4" s="1">
         <v>186100</v>
@@ -2190,7 +2184,7 @@
         <v>73</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="L4" s="6" t="s">
         <v>91</v>
@@ -2210,7 +2204,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>60</v>
@@ -2219,16 +2213,16 @@
         <v>60</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="G5" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>188</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>190</v>
       </c>
       <c r="I5" s="1">
         <v>186100</v>
@@ -2237,7 +2231,7 @@
         <v>73</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="L5" s="6" t="s">
         <v>91</v>
@@ -2255,7 +2249,7 @@
         <v>161</v>
       </c>
       <c r="U5" s="1" t="s">
-        <v>217</v>
+        <v>254</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.3">
@@ -2263,7 +2257,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>60</v>
@@ -2272,16 +2266,16 @@
         <v>60</v>
       </c>
       <c r="E6" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>188</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>190</v>
       </c>
       <c r="I6" s="1">
         <v>186100</v>
@@ -2290,7 +2284,7 @@
         <v>73</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="L6" s="6" t="s">
         <v>91</v>
@@ -2308,7 +2302,7 @@
         <v>25</v>
       </c>
       <c r="U6" s="1" t="s">
-        <v>220</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.3">
@@ -2316,7 +2310,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>60</v>
@@ -2325,16 +2319,16 @@
         <v>60</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>188</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>190</v>
       </c>
       <c r="I7" s="1">
         <v>186100</v>
@@ -2343,7 +2337,7 @@
         <v>73</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="L7" s="6" t="s">
         <v>91</v>
@@ -2361,7 +2355,7 @@
         <v>25</v>
       </c>
       <c r="U7" s="1" t="s">
-        <v>219</v>
+        <v>182</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.3">
@@ -2369,7 +2363,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>60</v>
@@ -2378,16 +2372,16 @@
         <v>60</v>
       </c>
       <c r="E8" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="G8" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="H8" s="1" t="s">
         <v>188</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>190</v>
       </c>
       <c r="I8" s="1">
         <v>186100</v>
@@ -2396,7 +2390,7 @@
         <v>73</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="L8" s="6" t="s">
         <v>91</v>
@@ -2414,7 +2408,7 @@
         <v>28</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>218</v>
+        <v>255</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.3">
@@ -2422,7 +2416,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>60</v>
@@ -2431,16 +2425,16 @@
         <v>60</v>
       </c>
       <c r="E9" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="H9" s="1" t="s">
         <v>188</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>190</v>
       </c>
       <c r="I9" s="1">
         <v>186100</v>
@@ -2449,7 +2443,7 @@
         <v>73</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="L9" s="6" t="s">
         <v>91</v>
@@ -2469,7 +2463,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>60</v>
@@ -2478,23 +2472,23 @@
         <v>60</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1" t="s">
         <v>73</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="L10" s="6" t="s">
         <v>91</v>
@@ -2707,10 +2701,10 @@
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="F8" s="3" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="H8" s="1"/>
     </row>
@@ -2871,7 +2865,7 @@
         <v>33</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -2888,7 +2882,7 @@
         <v>34</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -2905,7 +2899,7 @@
         <v>34</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -3071,14 +3065,14 @@
         <v>75</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="1" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="K3" s="1"/>
       <c r="L3" s="6">
@@ -3324,7 +3318,7 @@
         <v>41</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -3344,7 +3338,7 @@
         <v>42</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -3364,7 +3358,7 @@
         <v>43</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -3384,7 +3378,7 @@
         <v>44</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -3404,7 +3398,7 @@
         <v>45</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3514,7 +3508,7 @@
         <v>41</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -3534,7 +3528,7 @@
         <v>42</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
@@ -3554,7 +3548,7 @@
         <v>43</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -3574,7 +3568,7 @@
         <v>44</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -3594,7 +3588,7 @@
         <v>45</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>
@@ -4038,16 +4032,16 @@
       </c>
       <c r="V2" s="5"/>
       <c r="W2" s="5" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="X2" s="9" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="Y2" s="9" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="Z2" s="9" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.3">
@@ -4176,13 +4170,13 @@
         <v>60</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>79</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>80</v>
@@ -4232,13 +4226,13 @@
         <v>60</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>79</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>80</v>
@@ -4288,13 +4282,13 @@
         <v>60</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>117</v>
@@ -4344,13 +4338,13 @@
         <v>60</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>117</v>
@@ -4514,31 +4508,31 @@
         <v>145</v>
       </c>
       <c r="Y1" s="17" t="s">
+        <v>175</v>
+      </c>
+      <c r="Z1" s="17" t="s">
         <v>176</v>
       </c>
-      <c r="Z1" s="17" t="s">
+      <c r="AA1" s="17" t="s">
         <v>177</v>
       </c>
-      <c r="AA1" s="17" t="s">
+      <c r="AB1" s="19" t="s">
+        <v>164</v>
+      </c>
+      <c r="AC1" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="AD1" s="19" t="s">
+        <v>162</v>
+      </c>
+      <c r="AE1" s="19" t="s">
+        <v>173</v>
+      </c>
+      <c r="AF1" s="19" t="s">
+        <v>174</v>
+      </c>
+      <c r="AG1" s="19" t="s">
         <v>178</v>
-      </c>
-      <c r="AB1" s="19" t="s">
-        <v>165</v>
-      </c>
-      <c r="AC1" s="19" t="s">
-        <v>166</v>
-      </c>
-      <c r="AD1" s="19" t="s">
-        <v>163</v>
-      </c>
-      <c r="AE1" s="19" t="s">
-        <v>174</v>
-      </c>
-      <c r="AF1" s="19" t="s">
-        <v>175</v>
-      </c>
-      <c r="AG1" s="19" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="2" spans="1:33" x14ac:dyDescent="0.3">
@@ -4594,7 +4588,7 @@
         <v>148</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="S2" s="1" t="s">
         <v>86</v>
@@ -4749,7 +4743,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>60</v>
@@ -4800,7 +4794,7 @@
         <v>161</v>
       </c>
       <c r="AA5" s="1" t="s">
-        <v>162</v>
+        <v>256</v>
       </c>
       <c r="AB5" s="1"/>
       <c r="AC5" s="1"/>
@@ -4814,7 +4808,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>60</v>
@@ -4879,7 +4873,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>60</v>
@@ -4944,7 +4938,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>60</v>
@@ -4995,7 +4989,7 @@
         <v>28</v>
       </c>
       <c r="AA8" s="1" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="AB8" s="1"/>
       <c r="AC8" s="1"/>
@@ -5009,7 +5003,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>60</v>
@@ -5068,7 +5062,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>60</v>
@@ -5127,7 +5121,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>60</v>
@@ -5186,7 +5180,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>60</v>
@@ -5245,7 +5239,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>60</v>
@@ -5293,13 +5287,13 @@
       <c r="Z13" s="3"/>
       <c r="AA13" s="1"/>
       <c r="AB13" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="AC13" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="AC13" s="1" t="s">
-        <v>168</v>
-      </c>
       <c r="AD13" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AE13" s="1"/>
       <c r="AF13" s="1"/>
@@ -5310,7 +5304,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>60</v>
@@ -5361,10 +5355,10 @@
       <c r="AC14" s="1"/>
       <c r="AD14" s="1"/>
       <c r="AE14" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="AF14" s="5" t="s">
         <v>180</v>
-      </c>
-      <c r="AF14" s="5" t="s">
-        <v>181</v>
       </c>
       <c r="AG14" s="1"/>
     </row>
@@ -5426,7 +5420,7 @@
       <c r="AE15" s="1"/>
       <c r="AF15" s="1"/>
       <c r="AG15" s="1" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="16" spans="1:33" x14ac:dyDescent="0.3">
@@ -5434,7 +5428,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>60</v>
@@ -5491,7 +5485,7 @@
         <v>161</v>
       </c>
       <c r="AG16" s="1" t="s">
-        <v>182</v>
+        <v>253</v>
       </c>
     </row>
     <row r="17" spans="1:33" x14ac:dyDescent="0.3">
@@ -5499,7 +5493,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>60</v>
@@ -5564,7 +5558,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>60</v>
@@ -5621,7 +5615,7 @@
         <v>25</v>
       </c>
       <c r="AG18" s="1" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="19" spans="1:33" x14ac:dyDescent="0.3">
@@ -5629,7 +5623,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>60</v>
@@ -5686,7 +5680,7 @@
         <v>28</v>
       </c>
       <c r="AG19" s="1" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
     </row>
     <row r="21" spans="1:33" x14ac:dyDescent="0.3">
@@ -5720,7 +5714,7 @@
     <row r="26" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A26" s="18"/>
       <c r="B26" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -5814,10 +5808,10 @@
         <v>98</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="T1" s="2" t="s">
         <v>100</v>
@@ -5838,10 +5832,10 @@
         <v>122</v>
       </c>
       <c r="Z1" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="AA1" s="2" t="s">
         <v>176</v>
-      </c>
-      <c r="AA1" s="2" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.3">
@@ -5849,25 +5843,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>188</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>190</v>
       </c>
       <c r="I2" s="1">
         <v>186100</v>
@@ -5876,32 +5870,32 @@
         <v>73</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="L2" s="6" t="s">
         <v>91</v>
       </c>
       <c r="M2" s="10" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="N2" s="8" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="O2" s="6" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="P2" s="8">
         <v>7858408019</v>
       </c>
       <c r="Q2" s="5"/>
       <c r="R2" s="5" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="S2" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="T2" s="8" t="s">
         <v>207</v>
-      </c>
-      <c r="T2" s="8" t="s">
-        <v>209</v>
       </c>
       <c r="U2" s="5" t="s">
         <v>105</v>
@@ -5913,16 +5907,16 @@
         <v>148</v>
       </c>
       <c r="X2" s="9" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="Y2" s="9" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="Z2" s="9" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="AA2" s="9" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.3">
@@ -5930,7 +5924,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>60</v>
@@ -5939,20 +5933,20 @@
         <v>60</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>85</v>
       </c>
       <c r="I3" s="5"/>
       <c r="J3" s="1" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="K3" s="1">
         <v>493364140</v>

</xml_diff>

<commit_message>
Updated and added new scenarios
</commit_message>
<xml_diff>
--- a/data/CPSUI_Automation_Data.xlsx
+++ b/data/CPSUI_Automation_Data.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AG53052\EclipseWorkspace\CPSUI_Automation\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AG53052\EclipseWorkspace\CPSUI_Automation\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22152" windowHeight="8340" tabRatio="786" activeTab="3"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="783" firstSheet="3" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="PhoneSearch" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
     <sheet name="GovtMemberContactInfPhone" sheetId="10" r:id="rId10"/>
     <sheet name="Govt_Mbr_Text_Mail_Email_Pref" sheetId="11" r:id="rId11"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="986" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1019" uniqueCount="276">
   <si>
     <t>Update and validate the phone number preferences</t>
   </si>
@@ -319,9 +319,6 @@
   </si>
   <si>
     <t>JOHN1@ANTHEM.COM</t>
-  </si>
-  <si>
-    <t>DO NOT MAIL Woodland Hlls ,CALIFORNIA ,UNITED STATES ,91367</t>
   </si>
   <si>
     <t>preferredMailingAddress</t>
@@ -409,9 +406,6 @@
     </r>
   </si>
   <si>
-    <t>04/08/2021 05:05 AM</t>
-  </si>
-  <si>
     <t>updatedDateAndTimeInMemberInformation</t>
   </si>
   <si>
@@ -496,9 +490,6 @@
     <t>AG53052</t>
   </si>
   <si>
-    <t>DO NOT MAIL ,Woodland Hlls ,CALIFORNIA ,UNITED STATES ,91367</t>
-  </si>
-  <si>
     <t>WGS User</t>
   </si>
   <si>
@@ -692,12 +683,6 @@
   </si>
   <si>
     <t>4/22/2021</t>
-  </si>
-  <si>
-    <t>WAWID062</t>
-  </si>
-  <si>
-    <t>04/19/2021</t>
   </si>
   <si>
     <t>04/05/2021</t>
@@ -794,12 +779,6 @@
     <t>702T93657</t>
   </si>
   <si>
-    <t>ROSSI03</t>
-  </si>
-  <si>
-    <t>VALENTINO03</t>
-  </si>
-  <si>
     <t>10/22/1934</t>
   </si>
   <si>
@@ -819,6 +798,84 @@
   </si>
   <si>
     <t>History Details: Please enter From Date and End Date within 1 year range.</t>
+  </si>
+  <si>
+    <t>8185555555</t>
+  </si>
+  <si>
+    <t>C/O DO NOT MAIL Woodland Hlls ,CALIFORNIA ,UNITED STATES ,91367-1141</t>
+  </si>
+  <si>
+    <t>01</t>
+  </si>
+  <si>
+    <t>PETER03</t>
+  </si>
+  <si>
+    <t>ANTONY03</t>
+  </si>
+  <si>
+    <t>3/14/2022</t>
+  </si>
+  <si>
+    <t>03/14/2022 06:16 AM</t>
+  </si>
+  <si>
+    <t>Update and validate all the preference options under Gender Identity Preference</t>
+  </si>
+  <si>
+    <t>JERRY</t>
+  </si>
+  <si>
+    <t>TOM</t>
+  </si>
+  <si>
+    <t>09/19/1980</t>
+  </si>
+  <si>
+    <t>284932</t>
+  </si>
+  <si>
+    <t>238T96854</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Update and validate all the preference options under Covered CA Termination Reporting </t>
+  </si>
+  <si>
+    <t>Opt-Out</t>
+  </si>
+  <si>
+    <t>Opt-In</t>
+  </si>
+  <si>
+    <t>03/14/2022</t>
+  </si>
+  <si>
+    <t>C/O DO NOT MAIL ,Woodland Hlls ,CALIFORNIA ,UNITED STATES ,91367-1141</t>
+  </si>
+  <si>
+    <t>038T53444</t>
+  </si>
+  <si>
+    <t>RICHARDINA SIT</t>
+  </si>
+  <si>
+    <t>01/12/1996</t>
+  </si>
+  <si>
+    <t>W40355</t>
+  </si>
+  <si>
+    <t>covCA_Value1</t>
+  </si>
+  <si>
+    <t>covCA_Value2</t>
+  </si>
+  <si>
+    <t>gender_Identity_values</t>
+  </si>
+  <si>
+    <t>Male; Female; Non-Binary;Transgender Male;Transgender Female;Other</t>
   </si>
 </sst>
 </file>
@@ -925,7 +982,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -974,6 +1031,24 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1281,7 +1356,7 @@
         <v>7</v>
       </c>
       <c r="F1" s="23" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -1318,7 +1393,7 @@
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -1331,7 +1406,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>1</v>
@@ -1365,7 +1440,7 @@
         <v>0</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>2</v>
@@ -1456,7 +1531,7 @@
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="21" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -1484,7 +1559,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="63.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="62.5546875" customWidth="1"/>
     <col min="3" max="3" width="13.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.21875" bestFit="1" customWidth="1"/>
@@ -1547,10 +1622,10 @@
         <v>5</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="P1" s="2" t="s">
         <v>6</v>
@@ -1559,13 +1634,13 @@
         <v>7</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="U1" s="2" t="s">
         <v>15</v>
@@ -1579,7 +1654,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>60</v>
@@ -1588,16 +1663,16 @@
         <v>60</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>188</v>
       </c>
       <c r="I2" s="1">
         <v>186100</v>
@@ -1606,7 +1681,7 @@
         <v>73</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="L2" s="6" t="s">
         <v>91</v>
@@ -1623,19 +1698,19 @@
       <c r="P2" s="5"/>
       <c r="Q2" s="5"/>
       <c r="R2" s="5" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="S2" s="9" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="T2" s="9" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="U2" s="9" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="V2" s="9" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.3">
@@ -1643,7 +1718,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>60</v>
@@ -1652,23 +1727,23 @@
         <v>60</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="1" t="s">
         <v>73</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="L3" s="6" t="s">
         <v>91</v>
@@ -1693,7 +1768,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>60</v>
@@ -1702,23 +1777,23 @@
         <v>60</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="I4" s="1"/>
       <c r="J4" s="1" t="s">
         <v>73</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="L4" s="6" t="s">
         <v>91</v>
@@ -1743,7 +1818,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>60</v>
@@ -1752,22 +1827,22 @@
         <v>60</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="I5" s="1"/>
       <c r="J5" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="K5" s="1">
+        <v>194</v>
+      </c>
+      <c r="K5" s="24">
         <v>245687858</v>
       </c>
       <c r="L5" s="6">
@@ -1793,7 +1868,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>60</v>
@@ -1802,22 +1877,22 @@
         <v>60</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="K6" s="1">
+        <v>194</v>
+      </c>
+      <c r="K6" s="24">
         <v>245687858</v>
       </c>
       <c r="L6" s="6">
@@ -1843,7 +1918,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>60</v>
@@ -1852,13 +1927,13 @@
         <v>60</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>85</v>
@@ -1868,7 +1943,7 @@
         <v>65</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="L7" s="6" t="s">
         <v>69</v>
@@ -1893,7 +1968,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>60</v>
@@ -1902,13 +1977,13 @@
         <v>60</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>85</v>
@@ -1918,7 +1993,7 @@
         <v>65</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="L8" s="6" t="s">
         <v>69</v>
@@ -1940,16 +2015,17 @@
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2019,31 +2095,31 @@
         <v>59</v>
       </c>
       <c r="M1" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="N1" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="O1" s="12" t="s">
         <v>135</v>
       </c>
-      <c r="N1" s="12" t="s">
+      <c r="P1" s="12" t="s">
         <v>136</v>
       </c>
-      <c r="O1" s="12" t="s">
+      <c r="Q1" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="P1" s="12" t="s">
+      <c r="R1" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="Q1" s="12" t="s">
-        <v>139</v>
-      </c>
-      <c r="R1" s="12" t="s">
-        <v>140</v>
-      </c>
       <c r="S1" s="17" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="T1" s="17" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="U1" s="17" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.3">
@@ -2051,7 +2127,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>60</v>
@@ -2060,23 +2136,23 @@
         <v>60</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>85</v>
       </c>
       <c r="I2" s="1"/>
       <c r="J2" s="1" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="L2" s="6">
         <v>20</v>
@@ -2088,14 +2164,14 @@
         <v>2010313141</v>
       </c>
       <c r="O2" s="5" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="P2" s="5"/>
       <c r="Q2" s="5" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="R2" s="20" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="S2" s="6"/>
       <c r="T2" s="6"/>
@@ -2106,7 +2182,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>60</v>
@@ -2115,16 +2191,16 @@
         <v>60</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>188</v>
       </c>
       <c r="I3" s="1">
         <v>186100</v>
@@ -2133,7 +2209,7 @@
         <v>73</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="L3" s="6" t="s">
         <v>91</v>
@@ -2145,10 +2221,10 @@
       <c r="Q3" s="5"/>
       <c r="R3" s="3"/>
       <c r="S3" s="6" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="T3" s="6" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="U3" s="6"/>
     </row>
@@ -2157,7 +2233,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>60</v>
@@ -2166,16 +2242,16 @@
         <v>60</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="H4" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>188</v>
       </c>
       <c r="I4" s="1">
         <v>186100</v>
@@ -2184,7 +2260,7 @@
         <v>73</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="L4" s="6" t="s">
         <v>91</v>
@@ -2204,7 +2280,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>60</v>
@@ -2213,16 +2289,16 @@
         <v>60</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="H5" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>188</v>
       </c>
       <c r="I5" s="1">
         <v>186100</v>
@@ -2231,7 +2307,7 @@
         <v>73</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="L5" s="6" t="s">
         <v>91</v>
@@ -2243,13 +2319,13 @@
       <c r="Q5" s="5"/>
       <c r="R5" s="3"/>
       <c r="S5" s="3" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="T5" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="U5" s="1" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.3">
@@ -2257,7 +2333,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>60</v>
@@ -2266,16 +2342,16 @@
         <v>60</v>
       </c>
       <c r="E6" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="H6" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>188</v>
       </c>
       <c r="I6" s="1">
         <v>186100</v>
@@ -2284,7 +2360,7 @@
         <v>73</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="L6" s="6" t="s">
         <v>91</v>
@@ -2310,7 +2386,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>60</v>
@@ -2319,16 +2395,16 @@
         <v>60</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="H7" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>188</v>
       </c>
       <c r="I7" s="1">
         <v>186100</v>
@@ -2337,7 +2413,7 @@
         <v>73</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="L7" s="6" t="s">
         <v>91</v>
@@ -2355,7 +2431,7 @@
         <v>25</v>
       </c>
       <c r="U7" s="1" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.3">
@@ -2363,7 +2439,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>60</v>
@@ -2372,16 +2448,16 @@
         <v>60</v>
       </c>
       <c r="E8" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="H8" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>188</v>
       </c>
       <c r="I8" s="1">
         <v>186100</v>
@@ -2390,7 +2466,7 @@
         <v>73</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="L8" s="6" t="s">
         <v>91</v>
@@ -2408,7 +2484,7 @@
         <v>28</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.3">
@@ -2416,7 +2492,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>60</v>
@@ -2425,16 +2501,16 @@
         <v>60</v>
       </c>
       <c r="E9" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="H9" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>188</v>
       </c>
       <c r="I9" s="1">
         <v>186100</v>
@@ -2443,7 +2519,7 @@
         <v>73</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="L9" s="6" t="s">
         <v>91</v>
@@ -2463,7 +2539,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>60</v>
@@ -2472,23 +2548,23 @@
         <v>60</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1" t="s">
         <v>73</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="L10" s="6" t="s">
         <v>91</v>
@@ -2505,24 +2581,24 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A14" s="15"/>
       <c r="B14" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A15" s="16"/>
       <c r="B15" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -2701,10 +2777,10 @@
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="F8" s="3" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="H8" s="1"/>
     </row>
@@ -2716,7 +2792,7 @@
         <v>17</v>
       </c>
       <c r="C9" s="22">
-        <v>6175057745</v>
+        <v>4043878724</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -2814,7 +2890,7 @@
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -2865,7 +2941,7 @@
         <v>33</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -2882,7 +2958,7 @@
         <v>34</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -2899,7 +2975,7 @@
         <v>34</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -3065,14 +3141,14 @@
         <v>75</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="1" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="K3" s="1"/>
       <c r="L3" s="6">
@@ -3255,12 +3331,12 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -3318,7 +3394,7 @@
         <v>41</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -3338,7 +3414,7 @@
         <v>42</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -3358,7 +3434,7 @@
         <v>43</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -3378,7 +3454,7 @@
         <v>44</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -3398,7 +3474,7 @@
         <v>45</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3508,7 +3584,7 @@
         <v>41</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -3528,7 +3604,7 @@
         <v>42</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
@@ -3548,7 +3624,7 @@
         <v>43</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -3568,7 +3644,7 @@
         <v>44</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -3588,7 +3664,7 @@
         <v>45</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
     </row>
   </sheetData>
@@ -3668,43 +3744,43 @@
         <v>59</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="N1" s="2" t="s">
         <v>93</v>
       </c>
       <c r="O1" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="P1" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="Q1" s="2" t="s">
-        <v>98</v>
-      </c>
       <c r="R1" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="S1" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="T1" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="V1" s="2" t="s">
-        <v>103</v>
-      </c>
       <c r="W1" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="X1" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="Y1" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="Z1" s="2" t="s">
         <v>15</v>
@@ -3751,19 +3827,19 @@
         <v>91</v>
       </c>
       <c r="M2" s="10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="N2" s="8" t="s">
         <v>94</v>
       </c>
       <c r="O2" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="P2" s="8">
-        <v>8185555555</v>
+        <v>251</v>
+      </c>
+      <c r="P2" s="8" t="s">
+        <v>250</v>
       </c>
       <c r="Q2" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="R2" s="5" t="s">
         <v>86</v>
@@ -3773,25 +3849,25 @@
       </c>
       <c r="T2" s="5"/>
       <c r="U2" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="V2" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="V2" s="5" t="s">
+      <c r="W2" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="W2" s="5" t="s">
-        <v>106</v>
-      </c>
       <c r="X2" s="9" t="s">
-        <v>120</v>
+        <v>256</v>
       </c>
       <c r="Y2" s="9" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="Z2" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="AA2" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.3">
@@ -3799,34 +3875,34 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="H3" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="5" t="s">
         <v>117</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>118</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>71</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="L3" s="6">
         <v>2</v>
@@ -3836,7 +3912,9 @@
       <c r="O3" s="6"/>
       <c r="P3" s="6"/>
       <c r="Q3" s="6"/>
-      <c r="R3" s="6"/>
+      <c r="R3" s="5" t="s">
+        <v>86</v>
+      </c>
       <c r="S3" s="6"/>
       <c r="T3" s="6"/>
       <c r="U3" s="6"/>
@@ -3847,14 +3925,19 @@
       <c r="Z3" s="6"/>
       <c r="AA3" s="6"/>
     </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="O5" s="8" t="s">
+        <v>252</v>
+      </c>
+    </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>
@@ -3932,19 +4015,19 @@
         <v>59</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="O1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="R1" s="2" t="s">
         <v>6</v>
@@ -3953,19 +4036,19 @@
         <v>7</v>
       </c>
       <c r="T1" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="W1" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="U1" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="V1" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="W1" s="2" t="s">
-        <v>134</v>
-      </c>
       <c r="X1" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Y1" s="2" t="s">
         <v>15</v>
@@ -3979,7 +4062,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>60</v>
@@ -4028,20 +4111,20 @@
       <c r="S2" s="5"/>
       <c r="T2" s="5"/>
       <c r="U2" s="11" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="V2" s="5"/>
       <c r="W2" s="5" t="s">
-        <v>215</v>
+        <v>105</v>
       </c>
       <c r="X2" s="9" t="s">
-        <v>216</v>
+        <v>266</v>
       </c>
       <c r="Y2" s="9" t="s">
-        <v>216</v>
+        <v>255</v>
       </c>
       <c r="Z2" s="9" t="s">
-        <v>216</v>
+        <v>255</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.3">
@@ -4049,7 +4132,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>60</v>
@@ -4058,25 +4141,25 @@
         <v>60</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="H3" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="5" t="s">
         <v>117</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>118</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>71</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="L3" s="6">
         <v>2</v>
@@ -4105,7 +4188,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>60</v>
@@ -4114,25 +4197,25 @@
         <v>60</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="H4" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="I4" s="5" t="s">
         <v>117</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>118</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>71</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="L4" s="6">
         <v>2</v>
@@ -4161,7 +4244,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>60</v>
@@ -4170,13 +4253,13 @@
         <v>60</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>79</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>80</v>
@@ -4217,7 +4300,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>60</v>
@@ -4226,13 +4309,13 @@
         <v>60</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>79</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>80</v>
@@ -4273,7 +4356,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>60</v>
@@ -4282,16 +4365,16 @@
         <v>60</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I7" s="6">
         <v>270000</v>
@@ -4329,7 +4412,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>60</v>
@@ -4338,16 +4421,16 @@
         <v>60</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I8" s="6">
         <v>270000</v>
@@ -4382,22 +4465,23 @@
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AG26"/>
+  <dimension ref="A1:AJ29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.6640625" bestFit="1" customWidth="1"/>
@@ -4432,9 +4516,12 @@
     <col min="30" max="30" width="44.44140625" bestFit="1" customWidth="1"/>
     <col min="31" max="32" width="27.109375" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="66.88671875" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="15.5546875" customWidth="1"/>
+    <col min="35" max="35" width="16.44140625" customWidth="1"/>
+    <col min="36" max="36" width="22.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -4472,156 +4559,168 @@
         <v>59</v>
       </c>
       <c r="M1" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="N1" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="O1" s="12" t="s">
         <v>135</v>
       </c>
-      <c r="N1" s="12" t="s">
+      <c r="P1" s="12" t="s">
         <v>136</v>
       </c>
-      <c r="O1" s="12" t="s">
+      <c r="Q1" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="P1" s="12" t="s">
+      <c r="R1" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="Q1" s="12" t="s">
+      <c r="S1" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="R1" s="12" t="s">
+      <c r="T1" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="U1" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="S1" s="13" t="s">
+      <c r="V1" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="T1" s="13" t="s">
+      <c r="W1" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="X1" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="Y1" s="17" t="s">
+        <v>172</v>
+      </c>
+      <c r="Z1" s="17" t="s">
+        <v>173</v>
+      </c>
+      <c r="AA1" s="17" t="s">
+        <v>174</v>
+      </c>
+      <c r="AB1" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="AC1" s="19" t="s">
+        <v>162</v>
+      </c>
+      <c r="AD1" s="19" t="s">
+        <v>159</v>
+      </c>
+      <c r="AE1" s="19" t="s">
+        <v>170</v>
+      </c>
+      <c r="AF1" s="19" t="s">
+        <v>171</v>
+      </c>
+      <c r="AG1" s="19" t="s">
+        <v>175</v>
+      </c>
+      <c r="AH1" s="19" t="s">
+        <v>272</v>
+      </c>
+      <c r="AI1" s="19" t="s">
+        <v>273</v>
+      </c>
+      <c r="AJ1" s="19" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="2" spans="1:36" s="33" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="29">
+        <v>1</v>
+      </c>
+      <c r="B2" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="C2" s="29" t="s">
+        <v>60</v>
+      </c>
+      <c r="D2" s="29" t="s">
+        <v>60</v>
+      </c>
+      <c r="E2" s="29" t="s">
+        <v>88</v>
+      </c>
+      <c r="F2" s="29" t="s">
+        <v>89</v>
+      </c>
+      <c r="G2" s="30" t="s">
+        <v>90</v>
+      </c>
+      <c r="H2" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="I2" s="29">
+        <v>174134</v>
+      </c>
+      <c r="J2" s="29" t="s">
+        <v>73</v>
+      </c>
+      <c r="K2" s="29" t="s">
+        <v>92</v>
+      </c>
+      <c r="L2" s="31" t="s">
+        <v>91</v>
+      </c>
+      <c r="M2" s="31" t="s">
+        <v>86</v>
+      </c>
+      <c r="N2" s="30">
+        <v>5139699786</v>
+      </c>
+      <c r="O2" s="30" t="s">
+        <v>103</v>
+      </c>
+      <c r="P2" s="30" t="s">
+        <v>145</v>
+      </c>
+      <c r="Q2" s="30" t="s">
         <v>146</v>
       </c>
-      <c r="U1" s="13" t="s">
-        <v>142</v>
-      </c>
-      <c r="V1" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="W1" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="X1" s="13" t="s">
-        <v>145</v>
-      </c>
-      <c r="Y1" s="17" t="s">
-        <v>175</v>
-      </c>
-      <c r="Z1" s="17" t="s">
-        <v>176</v>
-      </c>
-      <c r="AA1" s="17" t="s">
-        <v>177</v>
-      </c>
-      <c r="AB1" s="19" t="s">
-        <v>164</v>
-      </c>
-      <c r="AC1" s="19" t="s">
-        <v>165</v>
-      </c>
-      <c r="AD1" s="19" t="s">
-        <v>162</v>
-      </c>
-      <c r="AE1" s="19" t="s">
-        <v>173</v>
-      </c>
-      <c r="AF1" s="19" t="s">
-        <v>174</v>
-      </c>
-      <c r="AG1" s="19" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A2" s="1">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="I2" s="1">
-        <v>174134</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="L2" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="M2" s="6" t="s">
+      <c r="R2" s="32" t="s">
+        <v>212</v>
+      </c>
+      <c r="S2" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="N2" s="5">
-        <v>5139699786</v>
-      </c>
-      <c r="O2" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="P2" s="5" t="s">
+      <c r="T2" s="31" t="s">
+        <v>267</v>
+      </c>
+      <c r="U2" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="V2" s="31"/>
+      <c r="W2" s="31" t="s">
         <v>147</v>
       </c>
-      <c r="Q2" s="5" t="s">
+      <c r="X2" s="31" t="s">
         <v>148</v>
       </c>
-      <c r="R2" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="T2" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="U2" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="V2" s="6"/>
-      <c r="W2" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="X2" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="Y2" s="6"/>
-      <c r="Z2" s="6"/>
-      <c r="AA2" s="6"/>
-      <c r="AB2" s="1"/>
-      <c r="AC2" s="1"/>
-      <c r="AD2" s="1"/>
-      <c r="AE2" s="1"/>
-      <c r="AF2" s="1"/>
-      <c r="AG2" s="1"/>
-    </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="Y2" s="31"/>
+      <c r="Z2" s="31"/>
+      <c r="AA2" s="31"/>
+      <c r="AB2" s="29"/>
+      <c r="AC2" s="29"/>
+      <c r="AD2" s="29"/>
+      <c r="AE2" s="29"/>
+      <c r="AF2" s="29"/>
+      <c r="AG2" s="29"/>
+      <c r="AH2" s="29"/>
+      <c r="AI2" s="29"/>
+      <c r="AJ2" s="29"/>
+    </row>
+    <row r="3" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>60</v>
@@ -4666,10 +4765,10 @@
       <c r="W3" s="6"/>
       <c r="X3" s="6"/>
       <c r="Y3" s="6" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="Z3" s="6" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="AA3" s="6"/>
       <c r="AB3" s="1"/>
@@ -4678,13 +4777,16 @@
       <c r="AE3" s="1"/>
       <c r="AF3" s="1"/>
       <c r="AG3" s="1"/>
-    </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="AH3" s="1"/>
+      <c r="AI3" s="1"/>
+      <c r="AJ3" s="1"/>
+    </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>60</v>
@@ -4693,25 +4795,25 @@
         <v>60</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="H4" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="I4" s="5" t="s">
         <v>117</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>118</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>71</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="L4" s="6">
         <v>2</v>
@@ -4737,13 +4839,16 @@
       <c r="AE4" s="1"/>
       <c r="AF4" s="1"/>
       <c r="AG4" s="1"/>
-    </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="AH4" s="1"/>
+      <c r="AI4" s="1"/>
+      <c r="AJ4" s="1"/>
+    </row>
+    <row r="5" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>60</v>
@@ -4788,13 +4893,13 @@
       <c r="W5" s="6"/>
       <c r="X5" s="6"/>
       <c r="Y5" s="3" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="Z5" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="AA5" s="1" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="AB5" s="1"/>
       <c r="AC5" s="1"/>
@@ -4802,13 +4907,16 @@
       <c r="AE5" s="1"/>
       <c r="AF5" s="1"/>
       <c r="AG5" s="1"/>
-    </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="AH5" s="1"/>
+      <c r="AI5" s="1"/>
+      <c r="AJ5" s="1"/>
+    </row>
+    <row r="6" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>60</v>
@@ -4867,13 +4975,16 @@
       <c r="AE6" s="1"/>
       <c r="AF6" s="1"/>
       <c r="AG6" s="1"/>
-    </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="AH6" s="1"/>
+      <c r="AI6" s="1"/>
+      <c r="AJ6" s="1"/>
+    </row>
+    <row r="7" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>60</v>
@@ -4932,13 +5043,16 @@
       <c r="AE7" s="1"/>
       <c r="AF7" s="1"/>
       <c r="AG7" s="1"/>
-    </row>
-    <row r="8" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="AH7" s="1"/>
+      <c r="AI7" s="1"/>
+      <c r="AJ7" s="1"/>
+    </row>
+    <row r="8" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>60</v>
@@ -4989,7 +5103,7 @@
         <v>28</v>
       </c>
       <c r="AA8" s="1" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="AB8" s="1"/>
       <c r="AC8" s="1"/>
@@ -4997,13 +5111,16 @@
       <c r="AE8" s="1"/>
       <c r="AF8" s="1"/>
       <c r="AG8" s="1"/>
-    </row>
-    <row r="9" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="AH8" s="1"/>
+      <c r="AI8" s="1"/>
+      <c r="AJ8" s="1"/>
+    </row>
+    <row r="9" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>60</v>
@@ -5011,29 +5128,29 @@
       <c r="D9" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E9" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="I9" s="1">
-        <v>174134</v>
-      </c>
-      <c r="J9" s="1" t="s">
+      <c r="E9" s="34" t="s">
+        <v>113</v>
+      </c>
+      <c r="F9" s="34" t="s">
+        <v>269</v>
+      </c>
+      <c r="G9" s="35" t="s">
+        <v>270</v>
+      </c>
+      <c r="H9" s="34" t="s">
+        <v>116</v>
+      </c>
+      <c r="I9" s="31" t="s">
+        <v>271</v>
+      </c>
+      <c r="J9" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="K9" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="L9" s="6" t="s">
-        <v>91</v>
+      <c r="K9" s="34" t="s">
+        <v>268</v>
+      </c>
+      <c r="L9" s="31" t="s">
+        <v>81</v>
       </c>
       <c r="M9" s="6"/>
       <c r="N9" s="6"/>
@@ -5056,13 +5173,16 @@
       <c r="AE9" s="1"/>
       <c r="AF9" s="1"/>
       <c r="AG9" s="1"/>
-    </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="AH9" s="1"/>
+      <c r="AI9" s="1"/>
+      <c r="AJ9" s="1"/>
+    </row>
+    <row r="10" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>60</v>
@@ -5071,25 +5191,25 @@
         <v>60</v>
       </c>
       <c r="E10" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="H10" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="I10" s="5" t="s">
         <v>117</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>118</v>
       </c>
       <c r="J10" s="1" t="s">
         <v>71</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="L10" s="6">
         <v>2</v>
@@ -5115,72 +5235,78 @@
       <c r="AE10" s="1"/>
       <c r="AF10" s="1"/>
       <c r="AG10" s="1"/>
-    </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A11" s="1">
+      <c r="AH10" s="1"/>
+      <c r="AI10" s="1"/>
+      <c r="AJ10" s="1"/>
+    </row>
+    <row r="11" spans="1:36" s="37" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="34">
         <v>10</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="I11" s="1">
-        <v>174134</v>
-      </c>
-      <c r="J11" s="1" t="s">
+      <c r="B11" s="34" t="s">
+        <v>166</v>
+      </c>
+      <c r="C11" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="D11" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="E11" s="34" t="s">
+        <v>113</v>
+      </c>
+      <c r="F11" s="34" t="s">
+        <v>269</v>
+      </c>
+      <c r="G11" s="35" t="s">
+        <v>270</v>
+      </c>
+      <c r="H11" s="34" t="s">
+        <v>116</v>
+      </c>
+      <c r="I11" s="31" t="s">
+        <v>271</v>
+      </c>
+      <c r="J11" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="K11" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="L11" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="M11" s="6"/>
-      <c r="N11" s="6"/>
-      <c r="O11" s="6"/>
-      <c r="P11" s="1"/>
-      <c r="Q11" s="1"/>
-      <c r="R11" s="1"/>
-      <c r="S11" s="1"/>
-      <c r="T11" s="6"/>
-      <c r="U11" s="6"/>
-      <c r="V11" s="6"/>
-      <c r="W11" s="6"/>
-      <c r="X11" s="6"/>
-      <c r="Y11" s="3"/>
-      <c r="Z11" s="3"/>
-      <c r="AA11" s="1"/>
-      <c r="AB11" s="1"/>
-      <c r="AC11" s="1"/>
-      <c r="AD11" s="1"/>
-      <c r="AE11" s="1"/>
-      <c r="AF11" s="1"/>
-      <c r="AG11" s="1"/>
-    </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="K11" s="34" t="s">
+        <v>268</v>
+      </c>
+      <c r="L11" s="31" t="s">
+        <v>81</v>
+      </c>
+      <c r="M11" s="31"/>
+      <c r="N11" s="31"/>
+      <c r="O11" s="31"/>
+      <c r="P11" s="34"/>
+      <c r="Q11" s="34"/>
+      <c r="R11" s="34"/>
+      <c r="S11" s="34"/>
+      <c r="T11" s="31"/>
+      <c r="U11" s="31"/>
+      <c r="V11" s="31"/>
+      <c r="W11" s="31"/>
+      <c r="X11" s="31"/>
+      <c r="Y11" s="36"/>
+      <c r="Z11" s="36"/>
+      <c r="AA11" s="34"/>
+      <c r="AB11" s="34"/>
+      <c r="AC11" s="34"/>
+      <c r="AD11" s="34"/>
+      <c r="AE11" s="34"/>
+      <c r="AF11" s="34"/>
+      <c r="AG11" s="34"/>
+      <c r="AH11" s="34"/>
+      <c r="AI11" s="34"/>
+      <c r="AJ11" s="34"/>
+    </row>
+    <row r="12" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>60</v>
@@ -5189,25 +5315,25 @@
         <v>60</v>
       </c>
       <c r="E12" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="H12" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="H12" s="1" t="s">
+      <c r="I12" s="5" t="s">
         <v>117</v>
-      </c>
-      <c r="I12" s="5" t="s">
-        <v>118</v>
       </c>
       <c r="J12" s="1" t="s">
         <v>71</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="L12" s="6">
         <v>2</v>
@@ -5233,78 +5359,84 @@
       <c r="AE12" s="1"/>
       <c r="AF12" s="1"/>
       <c r="AG12" s="1"/>
-    </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A13" s="1">
+      <c r="AH12" s="1"/>
+      <c r="AI12" s="1"/>
+      <c r="AJ12" s="1"/>
+    </row>
+    <row r="13" spans="1:36" s="37" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="34">
         <v>12</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="E13" s="1" t="s">
+      <c r="B13" s="34" t="s">
+        <v>165</v>
+      </c>
+      <c r="C13" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="D13" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="E13" s="34" t="s">
         <v>88</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="F13" s="34" t="s">
         <v>89</v>
       </c>
-      <c r="G13" s="5" t="s">
+      <c r="G13" s="35" t="s">
         <v>90</v>
       </c>
-      <c r="H13" s="1" t="s">
+      <c r="H13" s="34" t="s">
         <v>80</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="34">
         <v>174134</v>
       </c>
-      <c r="J13" s="1" t="s">
+      <c r="J13" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="K13" s="1" t="s">
+      <c r="K13" s="34" t="s">
         <v>92</v>
       </c>
-      <c r="L13" s="6" t="s">
+      <c r="L13" s="31" t="s">
         <v>91</v>
       </c>
-      <c r="M13" s="6"/>
-      <c r="N13" s="6"/>
-      <c r="O13" s="6"/>
-      <c r="P13" s="1"/>
-      <c r="Q13" s="1"/>
-      <c r="R13" s="1"/>
-      <c r="S13" s="1"/>
-      <c r="T13" s="6"/>
-      <c r="U13" s="6"/>
-      <c r="V13" s="6"/>
-      <c r="W13" s="6"/>
-      <c r="X13" s="6"/>
-      <c r="Y13" s="3"/>
-      <c r="Z13" s="3"/>
-      <c r="AA13" s="1"/>
-      <c r="AB13" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="AC13" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="AD13" s="1" t="s">
+      <c r="M13" s="31"/>
+      <c r="N13" s="31"/>
+      <c r="O13" s="31"/>
+      <c r="P13" s="34"/>
+      <c r="Q13" s="34"/>
+      <c r="R13" s="34"/>
+      <c r="S13" s="34"/>
+      <c r="T13" s="31"/>
+      <c r="U13" s="31"/>
+      <c r="V13" s="31"/>
+      <c r="W13" s="31"/>
+      <c r="X13" s="31"/>
+      <c r="Y13" s="36"/>
+      <c r="Z13" s="36"/>
+      <c r="AA13" s="34"/>
+      <c r="AB13" s="34" t="s">
         <v>163</v>
       </c>
-      <c r="AE13" s="1"/>
-      <c r="AF13" s="1"/>
-      <c r="AG13" s="1"/>
-    </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="AC13" s="34" t="s">
+        <v>164</v>
+      </c>
+      <c r="AD13" s="34" t="s">
+        <v>160</v>
+      </c>
+      <c r="AE13" s="34"/>
+      <c r="AF13" s="34"/>
+      <c r="AG13" s="34"/>
+      <c r="AH13" s="34"/>
+      <c r="AI13" s="34"/>
+      <c r="AJ13" s="34"/>
+    </row>
+    <row r="14" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>60</v>
@@ -5313,25 +5445,25 @@
         <v>60</v>
       </c>
       <c r="E14" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="G14" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="G14" s="5" t="s">
+      <c r="H14" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="I14" s="5" t="s">
         <v>117</v>
-      </c>
-      <c r="I14" s="5" t="s">
-        <v>118</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>71</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="L14" s="6">
         <v>2</v>
@@ -5355,19 +5487,22 @@
       <c r="AC14" s="1"/>
       <c r="AD14" s="1"/>
       <c r="AE14" s="5" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="AF14" s="5" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="AG14" s="1"/>
-    </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="AH14" s="1"/>
+      <c r="AI14" s="1"/>
+      <c r="AJ14" s="1"/>
+    </row>
+    <row r="15" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>60</v>
@@ -5376,25 +5511,25 @@
         <v>60</v>
       </c>
       <c r="E15" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="G15" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="G15" s="5" t="s">
+      <c r="H15" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="H15" s="1" t="s">
+      <c r="I15" s="5" t="s">
         <v>117</v>
-      </c>
-      <c r="I15" s="5" t="s">
-        <v>118</v>
       </c>
       <c r="J15" s="1" t="s">
         <v>71</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="L15" s="6">
         <v>2</v>
@@ -5420,15 +5555,18 @@
       <c r="AE15" s="1"/>
       <c r="AF15" s="1"/>
       <c r="AG15" s="1" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="16" spans="1:33" x14ac:dyDescent="0.3">
+        <v>178</v>
+      </c>
+      <c r="AH15" s="1"/>
+      <c r="AI15" s="1"/>
+      <c r="AJ15" s="1"/>
+    </row>
+    <row r="16" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>60</v>
@@ -5437,25 +5575,25 @@
         <v>60</v>
       </c>
       <c r="E16" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="G16" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="G16" s="5" t="s">
+      <c r="H16" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="H16" s="1" t="s">
+      <c r="I16" s="5" t="s">
         <v>117</v>
-      </c>
-      <c r="I16" s="5" t="s">
-        <v>118</v>
       </c>
       <c r="J16" s="1" t="s">
         <v>71</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="L16" s="6">
         <v>2</v>
@@ -5479,21 +5617,24 @@
       <c r="AC16" s="1"/>
       <c r="AD16" s="1"/>
       <c r="AE16" s="1" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="AF16" s="1" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="AG16" s="1" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="17" spans="1:33" x14ac:dyDescent="0.3">
+        <v>246</v>
+      </c>
+      <c r="AH16" s="1"/>
+      <c r="AI16" s="1"/>
+      <c r="AJ16" s="1"/>
+    </row>
+    <row r="17" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>60</v>
@@ -5502,25 +5643,25 @@
         <v>60</v>
       </c>
       <c r="E17" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F17" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="G17" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="G17" s="5" t="s">
+      <c r="H17" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="H17" s="1" t="s">
+      <c r="I17" s="5" t="s">
         <v>117</v>
-      </c>
-      <c r="I17" s="5" t="s">
-        <v>118</v>
       </c>
       <c r="J17" s="1" t="s">
         <v>71</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="L17" s="6">
         <v>2</v>
@@ -5552,13 +5693,16 @@
       <c r="AG17" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="18" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="AH17" s="1"/>
+      <c r="AI17" s="1"/>
+      <c r="AJ17" s="1"/>
+    </row>
+    <row r="18" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>60</v>
@@ -5567,25 +5711,25 @@
         <v>60</v>
       </c>
       <c r="E18" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="G18" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="G18" s="5" t="s">
+      <c r="H18" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="H18" s="1" t="s">
+      <c r="I18" s="5" t="s">
         <v>117</v>
-      </c>
-      <c r="I18" s="5" t="s">
-        <v>118</v>
       </c>
       <c r="J18" s="1" t="s">
         <v>71</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="L18" s="6">
         <v>2</v>
@@ -5615,15 +5759,18 @@
         <v>25</v>
       </c>
       <c r="AG18" s="1" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="19" spans="1:33" x14ac:dyDescent="0.3">
+        <v>179</v>
+      </c>
+      <c r="AH18" s="1"/>
+      <c r="AI18" s="1"/>
+      <c r="AJ18" s="1"/>
+    </row>
+    <row r="19" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>60</v>
@@ -5632,25 +5779,25 @@
         <v>60</v>
       </c>
       <c r="E19" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="G19" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="G19" s="5" t="s">
+      <c r="H19" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="H19" s="1" t="s">
+      <c r="I19" s="5" t="s">
         <v>117</v>
-      </c>
-      <c r="I19" s="5" t="s">
-        <v>118</v>
       </c>
       <c r="J19" s="1" t="s">
         <v>71</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="L19" s="6">
         <v>2</v>
@@ -5680,45 +5827,217 @@
         <v>28</v>
       </c>
       <c r="AG19" s="1" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="21" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B21" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="22" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B22" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="23" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A23" s="15"/>
-      <c r="B23" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="24" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A24" s="14"/>
+        <v>217</v>
+      </c>
+      <c r="AH19" s="1"/>
+      <c r="AI19" s="1"/>
+      <c r="AJ19" s="1"/>
+    </row>
+    <row r="20" spans="1:36" s="37" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="34">
+        <v>19</v>
+      </c>
+      <c r="B20" s="34" t="s">
+        <v>263</v>
+      </c>
+      <c r="C20" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="D20" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="E20" s="34" t="s">
+        <v>258</v>
+      </c>
+      <c r="F20" s="34" t="s">
+        <v>259</v>
+      </c>
+      <c r="G20" s="35" t="s">
+        <v>260</v>
+      </c>
+      <c r="H20" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="I20" s="35" t="s">
+        <v>261</v>
+      </c>
+      <c r="J20" s="34" t="s">
+        <v>73</v>
+      </c>
+      <c r="K20" s="34" t="s">
+        <v>262</v>
+      </c>
+      <c r="L20" s="31" t="s">
+        <v>91</v>
+      </c>
+      <c r="M20" s="31"/>
+      <c r="N20" s="35"/>
+      <c r="O20" s="35"/>
+      <c r="P20" s="35"/>
+      <c r="Q20" s="35"/>
+      <c r="R20" s="36"/>
+      <c r="S20" s="34"/>
+      <c r="T20" s="31"/>
+      <c r="U20" s="31"/>
+      <c r="V20" s="31"/>
+      <c r="W20" s="31"/>
+      <c r="X20" s="31"/>
+      <c r="Y20" s="36"/>
+      <c r="Z20" s="36"/>
+      <c r="AA20" s="34"/>
+      <c r="AB20" s="34"/>
+      <c r="AC20" s="34"/>
+      <c r="AD20" s="34"/>
+      <c r="AE20" s="34"/>
+      <c r="AF20" s="34"/>
+      <c r="AG20" s="34"/>
+      <c r="AH20" s="34" t="s">
+        <v>264</v>
+      </c>
+      <c r="AI20" s="34" t="s">
+        <v>265</v>
+      </c>
+      <c r="AJ20" s="34"/>
+    </row>
+    <row r="21" spans="1:36" s="37" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="34">
+        <v>20</v>
+      </c>
+      <c r="B21" s="34" t="s">
+        <v>257</v>
+      </c>
+      <c r="C21" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="D21" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="E21" s="34" t="s">
+        <v>258</v>
+      </c>
+      <c r="F21" s="34" t="s">
+        <v>259</v>
+      </c>
+      <c r="G21" s="35" t="s">
+        <v>260</v>
+      </c>
+      <c r="H21" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="I21" s="35" t="s">
+        <v>261</v>
+      </c>
+      <c r="J21" s="34" t="s">
+        <v>73</v>
+      </c>
+      <c r="K21" s="34" t="s">
+        <v>262</v>
+      </c>
+      <c r="L21" s="31" t="s">
+        <v>91</v>
+      </c>
+      <c r="M21" s="31"/>
+      <c r="N21" s="35"/>
+      <c r="O21" s="35"/>
+      <c r="P21" s="35"/>
+      <c r="Q21" s="35"/>
+      <c r="R21" s="36"/>
+      <c r="S21" s="34"/>
+      <c r="T21" s="31"/>
+      <c r="U21" s="31"/>
+      <c r="V21" s="31"/>
+      <c r="W21" s="31"/>
+      <c r="X21" s="31"/>
+      <c r="Y21" s="36"/>
+      <c r="Z21" s="36"/>
+      <c r="AA21" s="34"/>
+      <c r="AB21" s="34"/>
+      <c r="AC21" s="34"/>
+      <c r="AD21" s="34"/>
+      <c r="AE21" s="34"/>
+      <c r="AF21" s="34"/>
+      <c r="AG21" s="34"/>
+      <c r="AH21" s="34"/>
+      <c r="AI21" s="34"/>
+      <c r="AJ21" s="34" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="22" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A22" s="25"/>
+      <c r="B22" s="25"/>
+      <c r="C22" s="25"/>
+      <c r="D22" s="25"/>
+      <c r="E22" s="25"/>
+      <c r="F22" s="25"/>
+      <c r="G22" s="26"/>
+      <c r="H22" s="27"/>
+      <c r="I22" s="28"/>
+      <c r="J22" s="25"/>
+      <c r="K22" s="25"/>
+      <c r="L22" s="10"/>
+      <c r="M22" s="10"/>
+      <c r="N22" s="28"/>
+      <c r="O22" s="28"/>
+      <c r="P22" s="28"/>
+      <c r="Q22" s="28"/>
+      <c r="R22" s="26"/>
+      <c r="S22" s="25"/>
+      <c r="T22" s="10"/>
+      <c r="U22" s="10"/>
+      <c r="V22" s="10"/>
+      <c r="W22" s="10"/>
+      <c r="X22" s="10"/>
+      <c r="Y22" s="26"/>
+      <c r="Z22" s="26"/>
+      <c r="AA22" s="25"/>
+      <c r="AB22" s="25"/>
+      <c r="AC22" s="25"/>
+      <c r="AD22" s="25"/>
+      <c r="AE22" s="25"/>
+      <c r="AF22" s="25"/>
+      <c r="AG22" s="25"/>
+      <c r="AH22" s="25"/>
+      <c r="AI22" s="25"/>
+      <c r="AJ22" s="25"/>
+    </row>
+    <row r="24" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="25" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="B25" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="26" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A26" s="15"/>
+      <c r="B26" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="27" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A27" s="14"/>
+      <c r="B27" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="28" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A28" s="16"/>
+      <c r="B28" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="25" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A25" s="16"/>
-      <c r="B25" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="26" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A26" s="18"/>
-      <c r="B26" t="s">
-        <v>170</v>
+    <row r="29" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A29" s="18"/>
+      <c r="B29" t="s">
+        <v>167</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -5793,49 +6112,49 @@
         <v>59</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="N1" s="2" t="s">
         <v>93</v>
       </c>
       <c r="O1" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="P1" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="Q1" s="2" t="s">
-        <v>98</v>
-      </c>
       <c r="R1" s="2" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="U1" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="V1" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="V1" s="2" t="s">
-        <v>103</v>
-      </c>
       <c r="W1" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="X1" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="Y1" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="Z1" s="2" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="AA1" s="2" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.3">
@@ -5843,25 +6162,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="E2" s="1" t="s">
+      <c r="G2" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>188</v>
       </c>
       <c r="I2" s="1">
         <v>186100</v>
@@ -5870,53 +6189,53 @@
         <v>73</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="L2" s="6" t="s">
         <v>91</v>
       </c>
       <c r="M2" s="10" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="N2" s="8" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="O2" s="6" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="P2" s="8">
         <v>7858408019</v>
       </c>
       <c r="Q2" s="5"/>
       <c r="R2" s="5" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="S2" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="T2" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="U2" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="V2" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="W2" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="X2" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="T2" s="8" t="s">
-        <v>207</v>
-      </c>
-      <c r="U2" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="V2" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="W2" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="X2" s="9" t="s">
-        <v>208</v>
-      </c>
       <c r="Y2" s="9" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="Z2" s="9" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="AA2" s="9" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.3">
@@ -5924,7 +6243,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>60</v>
@@ -5933,20 +6252,20 @@
         <v>60</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>85</v>
       </c>
       <c r="I3" s="5"/>
       <c r="J3" s="1" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="K3" s="1">
         <v>493364140</v>
@@ -5972,12 +6291,12 @@
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>